<commit_message>
feat(sprint-1): add data quality assessment
- Create Data_Quality_Check worksheet
- Add missing value analysis
- Add duplicate checking summary
- Add data quality status indicators
- Prepare dataset for pivot table analysis
</commit_message>
<xml_diff>
--- a/data/raw/Graduate_Education_Market_Analytics.xlxs.xlsx
+++ b/data/raw/Graduate_Education_Market_Analytics.xlxs.xlsx
@@ -9,15 +9,16 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12330"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12330" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Raw_Data" sheetId="1" r:id="rId1"/>
-    <sheet name="Lookup" sheetId="6" r:id="rId2"/>
-    <sheet name="Data_Dictionary" sheetId="2" r:id="rId3"/>
-    <sheet name="Data_Quality_Log" sheetId="3" r:id="rId4"/>
-    <sheet name="Cleaning_Log" sheetId="4" r:id="rId5"/>
-    <sheet name="README" sheetId="5" r:id="rId6"/>
+    <sheet name="Data_Quality_Check" sheetId="8" r:id="rId2"/>
+    <sheet name="Lookup" sheetId="6" r:id="rId3"/>
+    <sheet name="Data_Dictionary" sheetId="2" r:id="rId4"/>
+    <sheet name="Data_Quality_Log" sheetId="3" r:id="rId5"/>
+    <sheet name="Cleaning_Log" sheetId="4" r:id="rId6"/>
+    <sheet name="README" sheetId="5" r:id="rId7"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -29,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="447" uniqueCount="217">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="457" uniqueCount="233">
   <si>
     <t>University</t>
   </si>
@@ -58,9 +59,6 @@
     <t>Scholarship Coverage</t>
   </si>
   <si>
-    <t xml:space="preserve">Intership Available </t>
-  </si>
-  <si>
     <t>Notes</t>
   </si>
   <si>
@@ -497,9 +495,6 @@
   </si>
   <si>
     <t>Full / Partial Tuition</t>
-  </si>
-  <si>
-    <t>Unknown</t>
   </si>
   <si>
     <t>MBA (IS track)</t>
@@ -681,6 +676,60 @@
   </si>
   <si>
     <t>PhD</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>Duplicate check</t>
+  </si>
+  <si>
+    <t>Metric</t>
+  </si>
+  <si>
+    <t>Formula</t>
+  </si>
+  <si>
+    <t>Result</t>
+  </si>
+  <si>
+    <t>Total Programs</t>
+  </si>
+  <si>
+    <t>Missing Tuition</t>
+  </si>
+  <si>
+    <t>Missing Language</t>
+  </si>
+  <si>
+    <t>Duplicate Programs</t>
+  </si>
+  <si>
+    <t>Programs in South Korea</t>
+  </si>
+  <si>
+    <t>Programs in China</t>
+  </si>
+  <si>
+    <t>Missing Scholarship Name</t>
+  </si>
+  <si>
+    <t>Missing Internship</t>
+  </si>
+  <si>
+    <t>Missing QS Ranking</t>
+  </si>
+  <si>
+    <t>Average Tuition (USD)</t>
+  </si>
+  <si>
+    <t>Highest Tuition (USD)</t>
+  </si>
+  <si>
+    <t>Lowest Tuition (USD)</t>
+  </si>
+  <si>
+    <t>Intership Available</t>
   </si>
 </sst>
 </file>
@@ -778,7 +827,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -823,15 +872,21 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
@@ -840,17 +895,26 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="17">
+  <dxfs count="18">
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -916,25 +980,28 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="tblGraduatePrograms" displayName="tblGraduatePrograms" ref="A1:P25" totalsRowShown="0" dataDxfId="16" headerRowCellStyle="Normal" dataCellStyle="Normal">
-  <autoFilter ref="A1:P25"/>
-  <tableColumns count="16">
-    <tableColumn id="1" name="University" dataDxfId="15" dataCellStyle="Normal"/>
-    <tableColumn id="2" name="Country" dataDxfId="14" dataCellStyle="Normal"/>
-    <tableColumn id="3" name="City" dataDxfId="13" dataCellStyle="Normal"/>
-    <tableColumn id="16" name="Campus study" dataDxfId="12"/>
-    <tableColumn id="4" name="Program" dataDxfId="11" dataCellStyle="Normal"/>
-    <tableColumn id="5" name="Program Category" dataDxfId="10" dataCellStyle="Normal"/>
-    <tableColumn id="6" name="Discipline" dataDxfId="9" dataCellStyle="Normal"/>
-    <tableColumn id="7" name="Language" dataDxfId="8" dataCellStyle="Normal"/>
-    <tableColumn id="8" name="Duration (Years)" dataDxfId="7" dataCellStyle="Normal"/>
-    <tableColumn id="9" name="QS Ranking " dataDxfId="6" dataCellStyle="Normal"/>
-    <tableColumn id="10" name="Tuition USD" dataDxfId="5" dataCellStyle="Normal"/>
-    <tableColumn id="11" name="Scholarship Name" dataDxfId="4" dataCellStyle="Normal"/>
-    <tableColumn id="12" name="Scholarship Coverage" dataDxfId="3" dataCellStyle="Normal"/>
-    <tableColumn id="13" name="Intership Available " dataDxfId="2" dataCellStyle="Normal"/>
-    <tableColumn id="15" name="Notes" dataDxfId="1"/>
-    <tableColumn id="14" name="Data Source" dataDxfId="0" dataCellStyle="Normal"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="tblGraduatePrograms" displayName="tblGraduatePrograms" ref="A1:Q25" totalsRowShown="0" dataDxfId="17" headerRowCellStyle="Normal" dataCellStyle="Normal">
+  <autoFilter ref="A1:Q25"/>
+  <tableColumns count="17">
+    <tableColumn id="1" name="University" dataDxfId="16" dataCellStyle="Normal"/>
+    <tableColumn id="2" name="Country" dataDxfId="15" dataCellStyle="Normal"/>
+    <tableColumn id="3" name="City" dataDxfId="14" dataCellStyle="Normal"/>
+    <tableColumn id="16" name="Campus study" dataDxfId="13"/>
+    <tableColumn id="4" name="Program" dataDxfId="12" dataCellStyle="Normal"/>
+    <tableColumn id="5" name="Program Category" dataDxfId="11" dataCellStyle="Normal"/>
+    <tableColumn id="6" name="Discipline" dataDxfId="10" dataCellStyle="Normal"/>
+    <tableColumn id="7" name="Language" dataDxfId="9" dataCellStyle="Normal"/>
+    <tableColumn id="8" name="Duration (Years)" dataDxfId="8" dataCellStyle="Normal"/>
+    <tableColumn id="9" name="QS Ranking " dataDxfId="7" dataCellStyle="Normal"/>
+    <tableColumn id="10" name="Tuition USD" dataDxfId="6" dataCellStyle="Normal"/>
+    <tableColumn id="11" name="Scholarship Name" dataDxfId="5" dataCellStyle="Normal"/>
+    <tableColumn id="12" name="Scholarship Coverage" dataDxfId="4" dataCellStyle="Normal"/>
+    <tableColumn id="13" name="Intership Available" dataDxfId="3" dataCellStyle="Normal"/>
+    <tableColumn id="15" name="Notes" dataDxfId="2"/>
+    <tableColumn id="17" name="Data Source" dataDxfId="1"/>
+    <tableColumn id="14" name="Duplicate check" dataDxfId="0" dataCellStyle="Normal">
+      <calculatedColumnFormula>IF(COUNTIFS(tblGraduatePrograms[University],tblGraduatePrograms[[#This Row],[University]],tblGraduatePrograms[Program],tblGraduatePrograms[[#This Row],[Program]])&gt;1,"Duplicate","Unique")</calculatedColumnFormula>
+    </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1237,7 +1304,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:P30"/>
+  <dimension ref="A1:Q30"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26.85546875" style="6" customWidth="1"/>
@@ -1252,12 +1319,12 @@
     <col min="11" max="11" width="15.140625" style="6" customWidth="1"/>
     <col min="12" max="12" width="18.5703125" style="6" customWidth="1"/>
     <col min="13" max="13" width="21.42578125" style="6" customWidth="1"/>
-    <col min="14" max="15" width="19.7109375" style="6" customWidth="1"/>
-    <col min="16" max="16" width="18.85546875" style="6" customWidth="1"/>
-    <col min="17" max="16384" width="9.140625" style="6"/>
+    <col min="14" max="16" width="19.7109375" style="6" customWidth="1"/>
+    <col min="17" max="17" width="18.85546875" style="6" customWidth="1"/>
+    <col min="18" max="16384" width="9.140625" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" s="7" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:17" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1268,13 +1335,13 @@
         <v>2</v>
       </c>
       <c r="D1" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="E1" t="s">
         <v>3</v>
       </c>
       <c r="F1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G1" t="s">
         <v>4</v>
@@ -1283,7 +1350,7 @@
         <v>5</v>
       </c>
       <c r="I1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="J1" t="s">
         <v>6</v>
@@ -1292,45 +1359,48 @@
         <v>7</v>
       </c>
       <c r="L1" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="M1" t="s">
         <v>8</v>
       </c>
       <c r="N1" t="s">
+        <v>232</v>
+      </c>
+      <c r="O1" t="s">
         <v>9</v>
       </c>
-      <c r="O1" t="s">
-        <v>10</v>
-      </c>
       <c r="P1" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="2" spans="1:16" ht="114" customHeight="1" x14ac:dyDescent="0.25">
+        <v>143</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="2" spans="1:17" ht="114" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="12" t="s">
+        <v>150</v>
+      </c>
+      <c r="B2" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="C2" s="12" t="s">
+        <v>148</v>
+      </c>
+      <c r="D2" s="12" t="s">
         <v>151</v>
       </c>
-      <c r="B2" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="C2" s="12" t="s">
-        <v>149</v>
-      </c>
-      <c r="D2" s="12" t="s">
+      <c r="E2" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="F2" s="12" t="s">
+        <v>145</v>
+      </c>
+      <c r="G2" s="12" t="s">
         <v>152</v>
       </c>
-      <c r="E2" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="F2" s="12" t="s">
-        <v>146</v>
-      </c>
-      <c r="G2" s="12" t="s">
+      <c r="H2" s="12" t="s">
         <v>153</v>
-      </c>
-      <c r="H2" s="12" t="s">
-        <v>154</v>
       </c>
       <c r="I2" s="12">
         <v>2</v>
@@ -1340,45 +1410,47 @@
         <v>8993.85</v>
       </c>
       <c r="L2" s="12" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="M2" s="12" t="s">
-        <v>155</v>
-      </c>
-      <c r="N2" s="12" t="s">
-        <v>156</v>
-      </c>
+        <v>154</v>
+      </c>
+      <c r="N2" s="12"/>
       <c r="O2" s="12" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="P2" s="12" t="s">
+        <v>149</v>
+      </c>
+      <c r="Q2" s="12" t="str">
+        <f>IF(COUNTIFS(tblGraduatePrograms[University],tblGraduatePrograms[[#This Row],[University]],tblGraduatePrograms[Program],tblGraduatePrograms[[#This Row],[Program]])&gt;1,"Duplicate","Unique")</f>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="3" spans="1:17" ht="101.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="12" t="s">
         <v>150</v>
       </c>
-    </row>
-    <row r="3" spans="1:16" ht="101.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="12" t="s">
+      <c r="B3" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="C3" s="12" t="s">
+        <v>148</v>
+      </c>
+      <c r="D3" s="12" t="s">
         <v>151</v>
       </c>
-      <c r="B3" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="C3" s="12" t="s">
-        <v>149</v>
-      </c>
-      <c r="D3" s="12" t="s">
-        <v>152</v>
-      </c>
       <c r="E3" s="12" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F3" s="12" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="G3" s="12" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="H3" s="12" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="I3" s="12">
         <v>2</v>
@@ -1388,45 +1460,49 @@
         <v>30000</v>
       </c>
       <c r="L3" s="12" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="M3" s="12" t="s">
+        <v>154</v>
+      </c>
+      <c r="N3" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="O3" s="12" t="s">
+        <v>190</v>
+      </c>
+      <c r="P3" s="12" t="s">
+        <v>149</v>
+      </c>
+      <c r="Q3" s="12" t="str">
+        <f>IF(COUNTIFS(tblGraduatePrograms[University],tblGraduatePrograms[[#This Row],[University]],tblGraduatePrograms[Program],tblGraduatePrograms[[#This Row],[Program]])&gt;1,"Duplicate","Unique")</f>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="4" spans="1:17" ht="90" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="C4" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="D4" s="12" t="s">
+        <v>151</v>
+      </c>
+      <c r="E4" s="12" t="s">
         <v>155</v>
       </c>
-      <c r="N3" s="12" t="s">
-        <v>80</v>
-      </c>
-      <c r="O3" s="12" t="s">
-        <v>192</v>
-      </c>
-      <c r="P3" s="12" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="4" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="B4" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="C4" s="12" t="s">
-        <v>16</v>
-      </c>
-      <c r="D4" s="12" t="s">
-        <v>152</v>
-      </c>
-      <c r="E4" s="12" t="s">
-        <v>157</v>
-      </c>
       <c r="F4" s="12" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="G4" s="12" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="H4" s="12" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="I4" s="12">
         <v>2</v>
@@ -1436,43 +1512,45 @@
         <v>30000</v>
       </c>
       <c r="L4" s="13" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="M4" s="12" t="s">
-        <v>155</v>
-      </c>
-      <c r="N4" s="13" t="s">
-        <v>156</v>
-      </c>
+        <v>154</v>
+      </c>
+      <c r="N4" s="13"/>
       <c r="O4" s="12" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="P4" s="12"/>
-    </row>
-    <row r="5" spans="1:16" ht="101.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Q4" s="12" t="str">
+        <f>IF(COUNTIFS(tblGraduatePrograms[University],tblGraduatePrograms[[#This Row],[University]],tblGraduatePrograms[Program],tblGraduatePrograms[[#This Row],[Program]])&gt;1,"Duplicate","Unique")</f>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="5" spans="1:17" ht="101.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="13" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B5" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="C5" s="13" t="s">
-        <v>16</v>
-      </c>
       <c r="D5" s="12" t="s">
+        <v>151</v>
+      </c>
+      <c r="E5" s="13" t="s">
+        <v>160</v>
+      </c>
+      <c r="F5" s="12" t="s">
+        <v>145</v>
+      </c>
+      <c r="G5" s="12" t="s">
         <v>152</v>
       </c>
-      <c r="E5" s="13" t="s">
-        <v>162</v>
-      </c>
-      <c r="F5" s="12" t="s">
-        <v>146</v>
-      </c>
-      <c r="G5" s="12" t="s">
+      <c r="H5" s="12" t="s">
         <v>153</v>
-      </c>
-      <c r="H5" s="12" t="s">
-        <v>154</v>
       </c>
       <c r="I5" s="13">
         <v>2</v>
@@ -1482,43 +1560,45 @@
         <v>16700</v>
       </c>
       <c r="L5" s="13" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="M5" s="12" t="s">
-        <v>155</v>
-      </c>
-      <c r="N5" s="13" t="s">
-        <v>156</v>
-      </c>
+        <v>154</v>
+      </c>
+      <c r="N5" s="13"/>
       <c r="O5" s="12" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="P5" s="13"/>
-    </row>
-    <row r="6" spans="1:16" ht="100.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Q5" s="12" t="str">
+        <f>IF(COUNTIFS(tblGraduatePrograms[University],tblGraduatePrograms[[#This Row],[University]],tblGraduatePrograms[Program],tblGraduatePrograms[[#This Row],[Program]])&gt;1,"Duplicate","Unique")</f>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17" ht="100.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="12" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B6" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="C6" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="C6" s="13" t="s">
-        <v>16</v>
-      </c>
       <c r="D6" s="12" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="E6" s="12" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="F6" s="12" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="G6" s="12" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="H6" s="12" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="I6" s="12">
         <v>2</v>
@@ -1528,37 +1608,39 @@
         <v>17000</v>
       </c>
       <c r="L6" s="13" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="M6" s="12" t="s">
-        <v>155</v>
-      </c>
-      <c r="N6" s="13" t="s">
-        <v>156</v>
-      </c>
+        <v>154</v>
+      </c>
+      <c r="N6" s="13"/>
       <c r="O6" s="12" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="P6" s="12"/>
-    </row>
-    <row r="7" spans="1:16" ht="100.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Q6" s="12" t="str">
+        <f>IF(COUNTIFS(tblGraduatePrograms[University],tblGraduatePrograms[[#This Row],[University]],tblGraduatePrograms[Program],tblGraduatePrograms[[#This Row],[Program]])&gt;1,"Duplicate","Unique")</f>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="7" spans="1:17" ht="100.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="13" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B7" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="C7" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="C7" s="13" t="s">
-        <v>16</v>
-      </c>
       <c r="D7" s="12" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="E7" s="13" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="F7" s="12" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="G7" s="13"/>
       <c r="H7" s="13"/>
@@ -1570,37 +1652,41 @@
         <v>29340</v>
       </c>
       <c r="L7" s="13" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="M7" s="12" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="N7" s="13" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="O7" s="12" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="P7" s="13"/>
-    </row>
-    <row r="8" spans="1:16" ht="100.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Q7" s="12" t="str">
+        <f>IF(COUNTIFS(tblGraduatePrograms[University],tblGraduatePrograms[[#This Row],[University]],tblGraduatePrograms[Program],tblGraduatePrograms[[#This Row],[Program]])&gt;1,"Duplicate","Unique")</f>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="8" spans="1:17" ht="100.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="13" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B8" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="C8" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="C8" s="13" t="s">
-        <v>16</v>
-      </c>
       <c r="D8" s="12" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="E8" s="13" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="F8" s="12" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="G8" s="13"/>
       <c r="H8" s="13"/>
@@ -1612,40 +1698,44 @@
         <v>29340</v>
       </c>
       <c r="L8" s="13" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="M8" s="12" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="N8" s="13" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="O8" s="12" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="P8" s="13"/>
-    </row>
-    <row r="9" spans="1:16" ht="104.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Q8" s="12" t="str">
+        <f>IF(COUNTIFS(tblGraduatePrograms[University],tblGraduatePrograms[[#This Row],[University]],tblGraduatePrograms[Program],tblGraduatePrograms[[#This Row],[Program]])&gt;1,"Duplicate","Unique")</f>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="9" spans="1:17" ht="104.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="13" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B9" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="C9" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="C9" s="13" t="s">
-        <v>16</v>
-      </c>
       <c r="D9" s="12" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="E9" s="13" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="F9" s="13" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="G9" s="13" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="H9" s="13"/>
       <c r="I9" s="13">
@@ -1656,43 +1746,45 @@
         <v>10280</v>
       </c>
       <c r="L9" s="13" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="M9" s="12" t="s">
-        <v>155</v>
-      </c>
-      <c r="N9" s="13" t="s">
-        <v>156</v>
-      </c>
+        <v>154</v>
+      </c>
+      <c r="N9" s="13"/>
       <c r="O9" s="12" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="P9" s="13"/>
-    </row>
-    <row r="10" spans="1:16" ht="105.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Q9" s="12" t="str">
+        <f>IF(COUNTIFS(tblGraduatePrograms[University],tblGraduatePrograms[[#This Row],[University]],tblGraduatePrograms[Program],tblGraduatePrograms[[#This Row],[Program]])&gt;1,"Duplicate","Unique")</f>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="10" spans="1:17" ht="105.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="12" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B10" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="C10" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="C10" s="12" t="s">
-        <v>16</v>
-      </c>
       <c r="D10" s="12" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="E10" s="12" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="F10" s="12" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="G10" s="12" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H10" s="12" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="I10" s="12">
         <v>2</v>
@@ -1702,43 +1794,47 @@
         <v>35000</v>
       </c>
       <c r="L10" s="12" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="M10" s="12" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="N10" s="12" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="O10" s="12" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="P10" s="12"/>
-    </row>
-    <row r="11" spans="1:16" ht="90" x14ac:dyDescent="0.25">
+      <c r="Q10" s="12" t="str">
+        <f>IF(COUNTIFS(tblGraduatePrograms[University],tblGraduatePrograms[[#This Row],[University]],tblGraduatePrograms[Program],tblGraduatePrograms[[#This Row],[Program]])&gt;1,"Duplicate","Unique")</f>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="11" spans="1:17" ht="90" x14ac:dyDescent="0.25">
       <c r="A11" s="13" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B11" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="C11" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="C11" s="12" t="s">
-        <v>16</v>
-      </c>
       <c r="D11" s="12" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="E11" s="12" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="F11" s="12" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="G11" s="12" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="H11" s="12" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="I11" s="13"/>
       <c r="J11" s="13"/>
@@ -1746,41 +1842,45 @@
         <v>20000</v>
       </c>
       <c r="L11" s="12" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="M11" s="12" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="N11" s="13"/>
       <c r="O11" s="12" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="P11" s="13"/>
-    </row>
-    <row r="12" spans="1:16" ht="105" x14ac:dyDescent="0.25">
+      <c r="Q11" s="12" t="str">
+        <f>IF(COUNTIFS(tblGraduatePrograms[University],tblGraduatePrograms[[#This Row],[University]],tblGraduatePrograms[Program],tblGraduatePrograms[[#This Row],[Program]])&gt;1,"Duplicate","Unique")</f>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="12" spans="1:17" ht="105" x14ac:dyDescent="0.25">
       <c r="A12" s="13" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B12" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="C12" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="C12" s="12" t="s">
-        <v>16</v>
-      </c>
       <c r="D12" s="12" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="E12" s="12" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F12" s="12" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="G12" s="12" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="H12" s="12" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="I12" s="12">
         <v>2</v>
@@ -1790,41 +1890,43 @@
         <v>20000</v>
       </c>
       <c r="L12" s="13" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="M12" s="12" t="s">
-        <v>155</v>
-      </c>
-      <c r="N12" s="13" t="s">
-        <v>156</v>
-      </c>
+        <v>154</v>
+      </c>
+      <c r="N12" s="13"/>
       <c r="O12" s="12"/>
       <c r="P12" s="13"/>
-    </row>
-    <row r="13" spans="1:16" ht="105" x14ac:dyDescent="0.25">
+      <c r="Q12" s="12" t="str">
+        <f>IF(COUNTIFS(tblGraduatePrograms[University],tblGraduatePrograms[[#This Row],[University]],tblGraduatePrograms[Program],tblGraduatePrograms[[#This Row],[Program]])&gt;1,"Duplicate","Unique")</f>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="13" spans="1:17" ht="105" x14ac:dyDescent="0.25">
       <c r="A13" s="12" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B13" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="C13" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="C13" s="12" t="s">
-        <v>16</v>
-      </c>
       <c r="D13" s="12" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="E13" s="12" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="F13" s="12" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="G13" s="12" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="H13" s="12" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="I13" s="12">
         <v>2</v>
@@ -1834,41 +1936,43 @@
         <v>28000</v>
       </c>
       <c r="L13" s="13" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="M13" s="12" t="s">
-        <v>155</v>
-      </c>
-      <c r="N13" s="13" t="s">
-        <v>156</v>
-      </c>
+        <v>154</v>
+      </c>
+      <c r="N13" s="13"/>
       <c r="O13" s="12"/>
       <c r="P13" s="12"/>
-    </row>
-    <row r="14" spans="1:16" ht="68.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Q13" s="12" t="str">
+        <f>IF(COUNTIFS(tblGraduatePrograms[University],tblGraduatePrograms[[#This Row],[University]],tblGraduatePrograms[Program],tblGraduatePrograms[[#This Row],[Program]])&gt;1,"Duplicate","Unique")</f>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="14" spans="1:17" ht="68.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="13" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="B14" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="C14" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="C14" s="12" t="s">
-        <v>16</v>
-      </c>
       <c r="D14" s="12" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="E14" s="13" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="F14" s="12" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="G14" s="12" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="H14" s="12" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="I14" s="13">
         <v>2</v>
@@ -1878,37 +1982,41 @@
         <v>10200</v>
       </c>
       <c r="L14" s="13" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="M14" s="12" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="N14" s="13"/>
       <c r="O14" s="12"/>
       <c r="P14" s="13"/>
-    </row>
-    <row r="15" spans="1:16" ht="118.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Q14" s="12" t="str">
+        <f>IF(COUNTIFS(tblGraduatePrograms[University],tblGraduatePrograms[[#This Row],[University]],tblGraduatePrograms[Program],tblGraduatePrograms[[#This Row],[Program]])&gt;1,"Duplicate","Unique")</f>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="15" spans="1:17" ht="118.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="B15" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="B15" s="12" t="s">
+      <c r="C15" s="12" t="s">
         <v>15</v>
-      </c>
-      <c r="C15" s="12" t="s">
-        <v>16</v>
       </c>
       <c r="D15" s="12"/>
       <c r="E15" s="12" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="F15" s="12" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="G15" s="12" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="H15" s="12" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="I15" s="12">
         <v>2</v>
@@ -1918,39 +2026,43 @@
         <v>10200</v>
       </c>
       <c r="L15" s="12" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="M15" s="12" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="N15" s="12"/>
       <c r="O15" s="12" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="P15" s="12"/>
-    </row>
-    <row r="16" spans="1:16" ht="118.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Q15" s="12" t="str">
+        <f>IF(COUNTIFS(tblGraduatePrograms[University],tblGraduatePrograms[[#This Row],[University]],tblGraduatePrograms[Program],tblGraduatePrograms[[#This Row],[Program]])&gt;1,"Duplicate","Unique")</f>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="16" spans="1:17" ht="118.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="B16" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="B16" s="12" t="s">
+      <c r="C16" s="12" t="s">
         <v>15</v>
-      </c>
-      <c r="C16" s="12" t="s">
-        <v>16</v>
       </c>
       <c r="D16" s="12"/>
       <c r="E16" s="13" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="F16" s="12" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="G16" s="12" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="H16" s="12" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="I16" s="13">
         <v>2</v>
@@ -1960,39 +2072,43 @@
         <v>18630</v>
       </c>
       <c r="L16" s="12" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="M16" s="12" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="N16" s="12"/>
       <c r="O16" s="12" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="P16" s="13"/>
-    </row>
-    <row r="17" spans="1:16" ht="109.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Q16" s="12" t="str">
+        <f>IF(COUNTIFS(tblGraduatePrograms[University],tblGraduatePrograms[[#This Row],[University]],tblGraduatePrograms[Program],tblGraduatePrograms[[#This Row],[Program]])&gt;1,"Duplicate","Unique")</f>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="17" spans="1:17" ht="109.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="B17" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="B17" s="12" t="s">
+      <c r="C17" s="12" t="s">
         <v>15</v>
-      </c>
-      <c r="C17" s="12" t="s">
-        <v>16</v>
       </c>
       <c r="D17" s="12"/>
       <c r="E17" s="12" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="F17" s="12" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="G17" s="12" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="H17" s="12" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="I17" s="12">
         <v>2</v>
@@ -2002,39 +2118,43 @@
         <v>30000</v>
       </c>
       <c r="L17" s="12" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="M17" s="12" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="N17" s="12"/>
       <c r="O17" s="12" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="P17" s="12"/>
-    </row>
-    <row r="18" spans="1:16" ht="135" x14ac:dyDescent="0.25">
+      <c r="Q17" s="12" t="str">
+        <f>IF(COUNTIFS(tblGraduatePrograms[University],tblGraduatePrograms[[#This Row],[University]],tblGraduatePrograms[Program],tblGraduatePrograms[[#This Row],[Program]])&gt;1,"Duplicate","Unique")</f>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="18" spans="1:17" ht="135" x14ac:dyDescent="0.25">
       <c r="A18" s="12" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B18" s="12" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C18" s="12" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D18" s="12"/>
       <c r="E18" s="12" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F18" s="12" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G18" s="12" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="H18" s="12" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="I18" s="12">
         <v>2.5</v>
@@ -2044,37 +2164,41 @@
         <v>13540</v>
       </c>
       <c r="L18" s="12" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="M18" s="12" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="N18" s="12"/>
       <c r="O18" s="12"/>
       <c r="P18" s="12"/>
-    </row>
-    <row r="19" spans="1:16" ht="135" x14ac:dyDescent="0.25">
+      <c r="Q18" s="12" t="str">
+        <f>IF(COUNTIFS(tblGraduatePrograms[University],tblGraduatePrograms[[#This Row],[University]],tblGraduatePrograms[Program],tblGraduatePrograms[[#This Row],[Program]])&gt;1,"Duplicate","Unique")</f>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="19" spans="1:17" ht="135" x14ac:dyDescent="0.25">
       <c r="A19" s="12" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B19" s="12" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C19" s="12" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D19" s="12"/>
       <c r="E19" s="13" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="F19" s="12" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="G19" s="12" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="H19" s="13" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="I19" s="13">
         <v>3</v>
@@ -2084,37 +2208,41 @@
         <v>10100</v>
       </c>
       <c r="L19" s="12" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="M19" s="12" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="N19" s="13"/>
       <c r="O19" s="12"/>
       <c r="P19" s="13"/>
-    </row>
-    <row r="20" spans="1:16" ht="135" x14ac:dyDescent="0.25">
+      <c r="Q19" s="12" t="str">
+        <f>IF(COUNTIFS(tblGraduatePrograms[University],tblGraduatePrograms[[#This Row],[University]],tblGraduatePrograms[Program],tblGraduatePrograms[[#This Row],[Program]])&gt;1,"Duplicate","Unique")</f>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="20" spans="1:17" ht="135" x14ac:dyDescent="0.25">
       <c r="A20" s="12" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B20" s="12" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C20" s="12" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D20" s="12"/>
       <c r="E20" s="13" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="F20" s="12" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="G20" s="12" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="H20" s="13" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="I20" s="13">
         <v>3</v>
@@ -2124,39 +2252,43 @@
         <v>10100</v>
       </c>
       <c r="L20" s="12" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="M20" s="12" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="N20" s="13"/>
       <c r="O20" s="12"/>
       <c r="P20" s="13"/>
-    </row>
-    <row r="21" spans="1:16" ht="135" x14ac:dyDescent="0.25">
+      <c r="Q20" s="12" t="str">
+        <f>IF(COUNTIFS(tblGraduatePrograms[University],tblGraduatePrograms[[#This Row],[University]],tblGraduatePrograms[Program],tblGraduatePrograms[[#This Row],[Program]])&gt;1,"Duplicate","Unique")</f>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="21" spans="1:17" ht="135" x14ac:dyDescent="0.25">
       <c r="A21" s="12" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B21" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="C21" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="D21" s="12" t="s">
+        <v>178</v>
+      </c>
+      <c r="E21" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="C21" s="12" t="s">
-        <v>31</v>
-      </c>
-      <c r="D21" s="12" t="s">
-        <v>180</v>
-      </c>
-      <c r="E21" s="12" t="s">
-        <v>28</v>
-      </c>
       <c r="F21" s="12" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G21" s="12" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="H21" s="12" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="I21" s="12">
         <v>2.5</v>
@@ -2166,37 +2298,41 @@
         <v>43750</v>
       </c>
       <c r="L21" s="12" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="M21" s="12" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="N21" s="12"/>
       <c r="O21" s="12"/>
       <c r="P21" s="12"/>
-    </row>
-    <row r="22" spans="1:16" ht="75" x14ac:dyDescent="0.25">
+      <c r="Q21" s="12" t="str">
+        <f>IF(COUNTIFS(tblGraduatePrograms[University],tblGraduatePrograms[[#This Row],[University]],tblGraduatePrograms[Program],tblGraduatePrograms[[#This Row],[Program]])&gt;1,"Duplicate","Unique")</f>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="22" spans="1:17" ht="75" x14ac:dyDescent="0.25">
       <c r="A22" s="12" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B22" s="12" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C22" s="12" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D22" s="12"/>
       <c r="E22" s="12" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="F22" s="12" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="G22" s="12" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="H22" s="12" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="I22" s="12">
         <v>2</v>
@@ -2206,37 +2342,41 @@
         <v>39700</v>
       </c>
       <c r="L22" s="12" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="M22" s="12" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="N22" s="12"/>
       <c r="O22" s="12"/>
       <c r="P22" s="12"/>
-    </row>
-    <row r="23" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+      <c r="Q22" s="12" t="str">
+        <f>IF(COUNTIFS(tblGraduatePrograms[University],tblGraduatePrograms[[#This Row],[University]],tblGraduatePrograms[Program],tblGraduatePrograms[[#This Row],[Program]])&gt;1,"Duplicate","Unique")</f>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="23" spans="1:17" ht="30" x14ac:dyDescent="0.25">
       <c r="A23" s="12" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B23" s="12" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C23" s="12" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D23" s="12"/>
       <c r="E23" s="12" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F23" s="12" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="G23" s="12" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="H23" s="12" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="I23" s="12">
         <v>2</v>
@@ -2248,29 +2388,33 @@
       <c r="N23" s="12"/>
       <c r="O23" s="12"/>
       <c r="P23" s="12"/>
-    </row>
-    <row r="24" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+      <c r="Q23" s="12" t="str">
+        <f>IF(COUNTIFS(tblGraduatePrograms[University],tblGraduatePrograms[[#This Row],[University]],tblGraduatePrograms[Program],tblGraduatePrograms[[#This Row],[Program]])&gt;1,"Duplicate","Unique")</f>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="24" spans="1:17" ht="30" x14ac:dyDescent="0.25">
       <c r="A24" s="12" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B24" s="12" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C24" s="12" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D24" s="12"/>
       <c r="E24" s="12" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F24" s="12" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="G24" s="12" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="H24" s="12" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="I24" s="12">
         <v>2</v>
@@ -2282,29 +2426,33 @@
       <c r="N24" s="12"/>
       <c r="O24" s="12"/>
       <c r="P24" s="12"/>
-    </row>
-    <row r="25" spans="1:16" ht="135" x14ac:dyDescent="0.25">
+      <c r="Q24" s="12" t="str">
+        <f>IF(COUNTIFS(tblGraduatePrograms[University],tblGraduatePrograms[[#This Row],[University]],tblGraduatePrograms[Program],tblGraduatePrograms[[#This Row],[Program]])&gt;1,"Duplicate","Unique")</f>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="25" spans="1:17" ht="135" x14ac:dyDescent="0.25">
       <c r="A25" s="12" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B25" s="12" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C25" s="12" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D25" s="12"/>
       <c r="E25" s="12" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F25" s="12" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="G25" s="12" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="H25" s="12" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="I25" s="12">
         <v>2</v>
@@ -2314,16 +2462,20 @@
         <v>10100</v>
       </c>
       <c r="L25" s="12" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="M25" s="12" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="N25" s="12"/>
       <c r="O25" s="12"/>
       <c r="P25" s="12"/>
-    </row>
-    <row r="30" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q25" s="12" t="str">
+        <f>IF(COUNTIFS(tblGraduatePrograms[University],tblGraduatePrograms[[#This Row],[University]],tblGraduatePrograms[Program],tblGraduatePrograms[[#This Row],[Program]])&gt;1,"Duplicate","Unique")</f>
+        <v>Unique</v>
+      </c>
+    </row>
+    <row r="30" spans="1:17" x14ac:dyDescent="0.25">
       <c r="G30" s="14"/>
     </row>
   </sheetData>
@@ -2361,6 +2513,203 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D13"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="18.7109375" customWidth="1"/>
+    <col min="2" max="3" width="18" customWidth="1"/>
+    <col min="4" max="4" width="18.28515625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" s="23" t="s">
+        <v>217</v>
+      </c>
+      <c r="B1" s="23" t="s">
+        <v>218</v>
+      </c>
+      <c r="C1" s="25" t="s">
+        <v>219</v>
+      </c>
+      <c r="D1" s="23" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" s="12" t="s">
+        <v>220</v>
+      </c>
+      <c r="B2" s="12">
+        <f>COUNTA(tblGraduatePrograms[Program])</f>
+        <v>24</v>
+      </c>
+      <c r="C2" s="24"/>
+      <c r="D2" s="12" t="str">
+        <f>"✅ Updated"</f>
+        <v>✅ Updated</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="12" t="s">
+        <v>223</v>
+      </c>
+      <c r="B3" s="12">
+        <f>COUNTIF(tblGraduatePrograms[Duplicate check],"Duplicate")</f>
+        <v>0</v>
+      </c>
+      <c r="C3" s="24"/>
+      <c r="D3" s="12" t="str">
+        <f>IF(B3=0,"🟢 Excellent","🔴 Duplicate Found")</f>
+        <v>🟢 Excellent</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" s="12" t="s">
+        <v>221</v>
+      </c>
+      <c r="B4" s="12">
+        <f>COUNTBLANK(tblGraduatePrograms[Tuition USD])</f>
+        <v>2</v>
+      </c>
+      <c r="C4" s="24"/>
+      <c r="D4" s="12" t="str">
+        <f>IF(B4=0,"🟢 Complete","🟡 Need Update")</f>
+        <v>🟡 Need Update</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A5" s="12" t="s">
+        <v>226</v>
+      </c>
+      <c r="B5" s="12">
+        <f>COUNTBLANK(tblGraduatePrograms[Scholarship Name])</f>
+        <v>2</v>
+      </c>
+      <c r="C5" s="24"/>
+      <c r="D5" s="12" t="str">
+        <f>IF(B5=0,"🟢 Complete","🟡 Need Update")</f>
+        <v>🟡 Need Update</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" s="12" t="s">
+        <v>222</v>
+      </c>
+      <c r="B6" s="12">
+        <f>COUNTBLANK(tblGraduatePrograms[Language])</f>
+        <v>3</v>
+      </c>
+      <c r="C6" s="24"/>
+      <c r="D6" s="12" t="str">
+        <f>IF(B6=0,"🟢 Complete","🟡 Need Update")</f>
+        <v>🟡 Need Update</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" s="12" t="s">
+        <v>227</v>
+      </c>
+      <c r="B7" s="12">
+        <f>COUNTBLANK(tblGraduatePrograms[Intership Available])</f>
+        <v>20</v>
+      </c>
+      <c r="C7" s="24"/>
+      <c r="D7" s="12" t="str">
+        <f>IF(B7=0,"🟢 Complete","🟡 Need Verification")</f>
+        <v>🟡 Need Verification</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" s="12" t="s">
+        <v>228</v>
+      </c>
+      <c r="B8" s="12">
+        <f>COUNTBLANK(tblGraduatePrograms[[QS Ranking ]])</f>
+        <v>24</v>
+      </c>
+      <c r="C8" s="24"/>
+      <c r="D8" s="12" t="str">
+        <f>IF(B8=0,"🟢 Complete","🟡 Need Update")</f>
+        <v>🟡 Need Update</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A9" s="12" t="s">
+        <v>224</v>
+      </c>
+      <c r="B9" s="12">
+        <f>COUNTIF(tblGraduatePrograms[Country],"South Korea")</f>
+        <v>16</v>
+      </c>
+      <c r="C9" s="24"/>
+      <c r="D9" s="12" t="str">
+        <f>"✅ OK"</f>
+        <v>✅ OK</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" s="12" t="s">
+        <v>225</v>
+      </c>
+      <c r="B10" s="12">
+        <f>COUNTIF(tblGraduatePrograms[Country],"China")</f>
+        <v>8</v>
+      </c>
+      <c r="C10" s="24"/>
+      <c r="D10" s="12" t="str">
+        <f>"✅ OK"</f>
+        <v>✅ OK</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A11" s="12" t="s">
+        <v>229</v>
+      </c>
+      <c r="B11" s="26">
+        <f>AVERAGE(tblGraduatePrograms[Tuition USD])</f>
+        <v>21407.902272727271</v>
+      </c>
+      <c r="C11" s="24"/>
+      <c r="D11" s="12" t="str">
+        <f>"📊 Calculated"</f>
+        <v>📊 Calculated</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A12" s="12" t="s">
+        <v>230</v>
+      </c>
+      <c r="B12" s="26">
+        <f>MAX(tblGraduatePrograms[Tuition USD])</f>
+        <v>43750</v>
+      </c>
+      <c r="C12" s="24"/>
+      <c r="D12" s="12" t="str">
+        <f>"📊 Calculated"</f>
+        <v>📊 Calculated</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A13" s="12" t="s">
+        <v>231</v>
+      </c>
+      <c r="B13" s="12">
+        <f>MIN(tblGraduatePrograms[Tuition USD])</f>
+        <v>8993.85</v>
+      </c>
+      <c r="C13" s="24"/>
+      <c r="D13" s="12" t="str">
+        <f>"📊 Calculated"</f>
+        <v>📊 Calculated</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:T10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2375,12 +2724,12 @@
   <sheetData>
     <row r="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A1" s="18" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B1" s="18"/>
       <c r="C1" s="12"/>
       <c r="D1" s="18" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="E1" s="18"/>
       <c r="F1" s="12"/>
@@ -2393,273 +2742,273 @@
         <v>1</v>
       </c>
       <c r="K1" s="18"/>
-      <c r="L1" s="21"/>
-      <c r="M1" s="22" t="s">
+      <c r="L1" s="15"/>
+      <c r="M1" s="16" t="s">
         <v>8</v>
       </c>
-      <c r="N1" s="22"/>
-      <c r="O1" s="21"/>
-      <c r="P1" s="22" t="s">
+      <c r="N1" s="16"/>
+      <c r="O1" s="15"/>
+      <c r="P1" s="16" t="s">
+        <v>208</v>
+      </c>
+      <c r="Q1" s="16"/>
+      <c r="S1" s="17" t="s">
         <v>210</v>
       </c>
-      <c r="Q1" s="22"/>
-      <c r="S1" s="15" t="s">
-        <v>212</v>
-      </c>
-      <c r="T1" s="15"/>
+      <c r="T1" s="17"/>
     </row>
     <row r="2" spans="1:20" ht="45" x14ac:dyDescent="0.25">
       <c r="A2" s="12" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B2" s="12"/>
       <c r="C2" s="12"/>
       <c r="D2" s="12" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E2" s="12"/>
       <c r="F2" s="12"/>
       <c r="G2" s="12" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="H2" s="12"/>
       <c r="I2" s="12"/>
       <c r="J2" s="12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="K2" s="12"/>
-      <c r="L2" s="21"/>
-      <c r="M2" s="21" t="s">
-        <v>206</v>
-      </c>
-      <c r="N2" s="21"/>
-      <c r="O2" s="21"/>
-      <c r="P2" s="21" t="s">
-        <v>80</v>
-      </c>
-      <c r="Q2" s="21"/>
+      <c r="L2" s="15"/>
+      <c r="M2" s="15" t="s">
+        <v>204</v>
+      </c>
+      <c r="N2" s="15"/>
+      <c r="O2" s="15"/>
+      <c r="P2" s="15" t="s">
+        <v>79</v>
+      </c>
+      <c r="Q2" s="15"/>
       <c r="S2" s="6" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
     </row>
     <row r="3" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="12" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B3" s="12"/>
       <c r="C3" s="12"/>
       <c r="D3" s="12" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E3" s="12"/>
       <c r="F3" s="12"/>
       <c r="G3" s="12" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="H3" s="12"/>
       <c r="I3" s="12"/>
       <c r="J3" s="12" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="K3" s="12"/>
-      <c r="L3" s="21"/>
-      <c r="M3" s="21" t="s">
-        <v>207</v>
-      </c>
-      <c r="N3" s="21"/>
-      <c r="O3" s="21"/>
-      <c r="P3" s="21" t="s">
-        <v>211</v>
-      </c>
-      <c r="Q3" s="21"/>
+      <c r="L3" s="15"/>
+      <c r="M3" s="15" t="s">
+        <v>205</v>
+      </c>
+      <c r="N3" s="15"/>
+      <c r="O3" s="15"/>
+      <c r="P3" s="15" t="s">
+        <v>209</v>
+      </c>
+      <c r="Q3" s="15"/>
       <c r="S3" s="6" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
     </row>
     <row r="4" spans="1:20" ht="45" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="B4" s="12"/>
       <c r="C4" s="12"/>
       <c r="D4" s="12" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="E4" s="12"/>
       <c r="F4" s="12"/>
       <c r="G4" s="12" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="H4" s="12"/>
       <c r="I4" s="12"/>
       <c r="J4" s="12"/>
       <c r="K4" s="12"/>
-      <c r="L4" s="21"/>
-      <c r="M4" s="21" t="s">
-        <v>155</v>
-      </c>
-      <c r="N4" s="21"/>
-      <c r="O4" s="21"/>
-      <c r="P4" s="21"/>
-      <c r="Q4" s="21"/>
+      <c r="L4" s="15"/>
+      <c r="M4" s="15" t="s">
+        <v>154</v>
+      </c>
+      <c r="N4" s="15"/>
+      <c r="O4" s="15"/>
+      <c r="P4" s="15"/>
+      <c r="Q4" s="15"/>
       <c r="S4" s="3" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
     </row>
     <row r="5" spans="1:20" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="12" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="B5" s="12"/>
       <c r="C5" s="12"/>
       <c r="D5" s="12" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="E5" s="12"/>
       <c r="F5" s="12"/>
       <c r="G5" s="12" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="H5" s="12"/>
       <c r="I5" s="12"/>
       <c r="J5" s="12"/>
       <c r="K5" s="12"/>
-      <c r="L5" s="21"/>
-      <c r="M5" s="21" t="s">
-        <v>208</v>
-      </c>
-      <c r="N5" s="21"/>
-      <c r="O5" s="21"/>
-      <c r="P5" s="21"/>
-      <c r="Q5" s="21"/>
+      <c r="L5" s="15"/>
+      <c r="M5" s="15" t="s">
+        <v>206</v>
+      </c>
+      <c r="N5" s="15"/>
+      <c r="O5" s="15"/>
+      <c r="P5" s="15"/>
+      <c r="Q5" s="15"/>
       <c r="S5" s="3" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
     </row>
     <row r="6" spans="1:20" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="12" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="B6" s="12"/>
       <c r="C6" s="12"/>
       <c r="D6" s="12" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E6" s="12"/>
       <c r="F6" s="12"/>
       <c r="G6" s="12" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="H6" s="12"/>
       <c r="I6" s="12"/>
       <c r="J6" s="12"/>
       <c r="K6" s="12"/>
-      <c r="L6" s="21"/>
-      <c r="M6" s="21" t="s">
-        <v>209</v>
-      </c>
-      <c r="N6" s="21"/>
-      <c r="O6" s="21"/>
-      <c r="P6" s="21"/>
-      <c r="Q6" s="21"/>
+      <c r="L6" s="15"/>
+      <c r="M6" s="15" t="s">
+        <v>207</v>
+      </c>
+      <c r="N6" s="15"/>
+      <c r="O6" s="15"/>
+      <c r="P6" s="15"/>
+      <c r="Q6" s="15"/>
       <c r="S6" s="6" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
     </row>
     <row r="7" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A7" s="12" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="B7" s="12"/>
       <c r="C7" s="12"/>
       <c r="D7" s="12" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="E7" s="12"/>
       <c r="F7" s="12"/>
       <c r="G7" s="12" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="H7" s="12"/>
       <c r="I7" s="12"/>
       <c r="J7" s="12"/>
       <c r="K7" s="12"/>
-      <c r="L7" s="21"/>
-      <c r="M7" s="21"/>
-      <c r="N7" s="21"/>
-      <c r="O7" s="21"/>
-      <c r="P7" s="21"/>
-      <c r="Q7" s="21"/>
+      <c r="L7" s="15"/>
+      <c r="M7" s="15"/>
+      <c r="N7" s="15"/>
+      <c r="O7" s="15"/>
+      <c r="P7" s="15"/>
+      <c r="Q7" s="15"/>
       <c r="S7" s="6"/>
     </row>
     <row r="8" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A8" s="12" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="B8" s="12"/>
       <c r="C8" s="12"/>
       <c r="D8" s="12" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="E8" s="12"/>
       <c r="F8" s="12"/>
       <c r="G8" s="12" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="H8" s="12"/>
       <c r="I8" s="12"/>
       <c r="J8" s="12"/>
       <c r="K8" s="12"/>
-      <c r="L8" s="21"/>
-      <c r="M8" s="21"/>
-      <c r="N8" s="21"/>
-      <c r="O8" s="21"/>
-      <c r="P8" s="21"/>
-      <c r="Q8" s="21"/>
+      <c r="L8" s="15"/>
+      <c r="M8" s="15"/>
+      <c r="N8" s="15"/>
+      <c r="O8" s="15"/>
+      <c r="P8" s="15"/>
+      <c r="Q8" s="15"/>
       <c r="S8" s="3"/>
     </row>
     <row r="9" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A9" s="21"/>
-      <c r="B9" s="21"/>
-      <c r="C9" s="21"/>
-      <c r="D9" s="21" t="s">
-        <v>200</v>
-      </c>
-      <c r="E9" s="21"/>
-      <c r="F9" s="21"/>
-      <c r="G9" s="21"/>
-      <c r="H9" s="21"/>
-      <c r="I9" s="21"/>
-      <c r="J9" s="21"/>
-      <c r="K9" s="21"/>
-      <c r="L9" s="21"/>
-      <c r="M9" s="21"/>
-      <c r="N9" s="21"/>
-      <c r="O9" s="21"/>
-      <c r="P9" s="21"/>
-      <c r="Q9" s="21"/>
+      <c r="A9" s="15"/>
+      <c r="B9" s="15"/>
+      <c r="C9" s="15"/>
+      <c r="D9" s="15" t="s">
+        <v>198</v>
+      </c>
+      <c r="E9" s="15"/>
+      <c r="F9" s="15"/>
+      <c r="G9" s="15"/>
+      <c r="H9" s="15"/>
+      <c r="I9" s="15"/>
+      <c r="J9" s="15"/>
+      <c r="K9" s="15"/>
+      <c r="L9" s="15"/>
+      <c r="M9" s="15"/>
+      <c r="N9" s="15"/>
+      <c r="O9" s="15"/>
+      <c r="P9" s="15"/>
+      <c r="Q9" s="15"/>
       <c r="S9" s="6"/>
     </row>
     <row r="10" spans="1:20" ht="30" x14ac:dyDescent="0.25">
-      <c r="A10" s="21"/>
-      <c r="B10" s="21"/>
-      <c r="C10" s="21"/>
+      <c r="A10" s="15"/>
+      <c r="B10" s="15"/>
+      <c r="C10" s="15"/>
       <c r="D10" s="12" t="s">
-        <v>201</v>
-      </c>
-      <c r="E10" s="21"/>
-      <c r="F10" s="21"/>
-      <c r="G10" s="21"/>
-      <c r="H10" s="21"/>
-      <c r="I10" s="21"/>
-      <c r="J10" s="21"/>
-      <c r="K10" s="21"/>
-      <c r="L10" s="21"/>
-      <c r="M10" s="21"/>
-      <c r="N10" s="21"/>
-      <c r="O10" s="21"/>
-      <c r="P10" s="21"/>
-      <c r="Q10" s="21"/>
+        <v>199</v>
+      </c>
+      <c r="E10" s="15"/>
+      <c r="F10" s="15"/>
+      <c r="G10" s="15"/>
+      <c r="H10" s="15"/>
+      <c r="I10" s="15"/>
+      <c r="J10" s="15"/>
+      <c r="K10" s="15"/>
+      <c r="L10" s="15"/>
+      <c r="M10" s="15"/>
+      <c r="N10" s="15"/>
+      <c r="O10" s="15"/>
+      <c r="P10" s="15"/>
+      <c r="Q10" s="15"/>
       <c r="S10" s="6"/>
     </row>
   </sheetData>
@@ -2676,7 +3025,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:F15"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2692,22 +3041,22 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>42</v>
-      </c>
       <c r="E1" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="30" x14ac:dyDescent="0.25">
@@ -2715,19 +3064,19 @@
         <v>0</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="45" x14ac:dyDescent="0.25">
@@ -2735,19 +3084,19 @@
         <v>1</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="45" x14ac:dyDescent="0.25">
@@ -2755,19 +3104,19 @@
         <v>2</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="30" x14ac:dyDescent="0.25">
@@ -2775,39 +3124,39 @@
         <v>3</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D5" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="F5" s="2" t="s">
         <v>65</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="120" x14ac:dyDescent="0.25">
       <c r="A6" s="8" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="135" x14ac:dyDescent="0.25">
@@ -2815,19 +3164,19 @@
         <v>4</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D7" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="F7" s="2" t="s">
         <v>68</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="F7" s="2" t="s">
-        <v>69</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="30" x14ac:dyDescent="0.25">
@@ -2835,59 +3184,59 @@
         <v>5</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="8" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D9" s="4">
         <v>2</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C10" s="2" t="s">
         <v>44</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>45</v>
       </c>
       <c r="D10" s="4">
         <v>47</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="45" x14ac:dyDescent="0.25">
@@ -2895,39 +3244,39 @@
         <v>7</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D11" s="4">
         <v>6500</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="75" x14ac:dyDescent="0.25">
       <c r="A12" s="8" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D12" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="F12" s="2" t="s">
         <v>75</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>95</v>
-      </c>
-      <c r="F12" s="2" t="s">
-        <v>76</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="60" x14ac:dyDescent="0.25">
@@ -2935,71 +3284,62 @@
         <v>8</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D13" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="F13" s="2" t="s">
         <v>77</v>
-      </c>
-      <c r="E13" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="F13" s="2" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="B14" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="B14" s="2" t="s">
-        <v>60</v>
-      </c>
       <c r="C14" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="D14" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="D14" s="2" t="s">
+      <c r="E14" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="F14" s="2" t="s">
         <v>80</v>
-      </c>
-      <c r="E14" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="F14" s="2" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D15" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="F15" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="E15" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="F15" s="2" t="s">
-        <v>83</v>
-      </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -3015,6 +3355,15 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H51"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -3024,86 +3373,86 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="17" t="s">
-        <v>109</v>
-      </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
-      <c r="E1" s="17"/>
-      <c r="F1" s="17"/>
-      <c r="G1" s="17"/>
-      <c r="H1" s="17"/>
+      <c r="A1" s="20" t="s">
+        <v>108</v>
+      </c>
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="20"/>
+      <c r="E1" s="20"/>
+      <c r="F1" s="20"/>
+      <c r="G1" s="20"/>
+      <c r="H1" s="20"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="10"/>
       <c r="B2" s="10"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A3" s="19" t="s">
-        <v>135</v>
-      </c>
-      <c r="B3" s="19"/>
+      <c r="A3" s="21" t="s">
+        <v>134</v>
+      </c>
+      <c r="B3" s="21"/>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="B4" s="1" t="s">
         <v>121</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="B5" s="2" t="s">
         <v>110</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>111</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="B6" s="2" t="s">
         <v>112</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>113</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="B7" s="2" t="s">
         <v>114</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>115</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>116</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>117</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="B10" s="2" t="s">
         <v>119</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="18" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B13" s="18"/>
       <c r="C13" s="18"/>
@@ -3114,148 +3463,148 @@
       <c r="H13" s="18"/>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A18" s="20" t="s">
-        <v>136</v>
-      </c>
-      <c r="B18" s="20"/>
+      <c r="A18" s="22" t="s">
+        <v>135</v>
+      </c>
+      <c r="B18" s="22"/>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="B19" s="1" t="s">
         <v>100</v>
-      </c>
-      <c r="B19" s="1" t="s">
-        <v>101</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="21" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="22" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="24" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A28" s="20" t="s">
-        <v>137</v>
-      </c>
-      <c r="B28" s="20"/>
+      <c r="A28" s="22" t="s">
+        <v>136</v>
+      </c>
+      <c r="B28" s="22"/>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="B29" s="1" t="s">
         <v>128</v>
-      </c>
-      <c r="B29" s="1" t="s">
-        <v>129</v>
       </c>
     </row>
     <row r="30" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="B30" s="2" t="s">
         <v>130</v>
-      </c>
-      <c r="B30" s="2" t="s">
-        <v>131</v>
       </c>
     </row>
     <row r="31" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="B32" s="2" t="s">
         <v>133</v>
       </c>
-      <c r="B32" s="2" t="s">
-        <v>134</v>
-      </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A36" s="20" t="s">
-        <v>138</v>
-      </c>
-      <c r="B36" s="20"/>
+      <c r="A36" s="22" t="s">
+        <v>137</v>
+      </c>
+      <c r="B36" s="22"/>
     </row>
     <row r="37" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="B37" s="1" t="s">
         <v>128</v>
-      </c>
-      <c r="B37" s="1" t="s">
-        <v>129</v>
       </c>
       <c r="C37" s="9"/>
     </row>
     <row r="38" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="B38" s="2" t="s">
         <v>130</v>
-      </c>
-      <c r="B38" s="2" t="s">
-        <v>131</v>
       </c>
       <c r="C38" s="10"/>
     </row>
     <row r="39" spans="1:3" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C39" s="10"/>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="B40" s="2" t="s">
         <v>133</v>
       </c>
-      <c r="B40" s="2" t="s">
-        <v>134</v>
-      </c>
       <c r="C40" s="10"/>
     </row>
     <row r="45" spans="1:3" ht="18" x14ac:dyDescent="0.25">
-      <c r="A45" s="16" t="s">
-        <v>139</v>
-      </c>
-      <c r="B45" s="16"/>
+      <c r="A45" s="19" t="s">
+        <v>138</v>
+      </c>
+      <c r="B45" s="19"/>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.25">
@@ -3263,17 +3612,17 @@
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A49" s="11" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A50" s="11" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A51" s="11" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(sprint-1): create pivot table analysis
- Create Pivot Analysis worksheet
- Programs by Country
- Programs by Program Category
- Programs by Language
- Average Tuition by Country
- Format Pivot Tables
</commit_message>
<xml_diff>
--- a/data/raw/Graduate_Education_Market_Analytics.xlxs.xlsx
+++ b/data/raw/Graduate_Education_Market_Analytics.xlxs.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12330" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12330" activeTab="7"/>
   </bookViews>
   <sheets>
     <sheet name="Raw_Data" sheetId="1" r:id="rId1"/>
@@ -19,8 +19,12 @@
     <sheet name="Data_Quality_Log" sheetId="3" r:id="rId5"/>
     <sheet name="Cleaning_Log" sheetId="4" r:id="rId6"/>
     <sheet name="README" sheetId="5" r:id="rId7"/>
+    <sheet name="Pivot_Analysis" sheetId="9" r:id="rId8"/>
   </sheets>
   <calcPr calcId="162913"/>
+  <pivotCaches>
+    <pivotCache cacheId="10" r:id="rId9"/>
+  </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -30,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="457" uniqueCount="233">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="487" uniqueCount="240">
   <si>
     <t>University</t>
   </si>
@@ -558,9 +562,6 @@
   </si>
   <si>
     <t>Communication</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Chinese </t>
   </si>
   <si>
     <t>Information and Communication Engineering</t>
@@ -730,13 +731,37 @@
   </si>
   <si>
     <t>Intership Available</t>
+  </si>
+  <si>
+    <t>Grand Total</t>
+  </si>
+  <si>
+    <t>Count of Program</t>
+  </si>
+  <si>
+    <t>(blank)</t>
+  </si>
+  <si>
+    <t>Average of Tuition USD</t>
+  </si>
+  <si>
+    <t>Programs by Country</t>
+  </si>
+  <si>
+    <t>Programs by Category</t>
+  </si>
+  <si>
+    <t>Programs by Language</t>
+  </si>
+  <si>
+    <t>Average Tuition by Country</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -770,6 +795,12 @@
       <family val="2"/>
       <charset val="163"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color theme="4" tint="-0.499984740745262"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -827,7 +858,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -874,6 +905,18 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -895,23 +938,627 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="18">
+  <dxfs count="220">
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="0.000"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="0.0000"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="0.000"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="0.000"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="0.000"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="0.0000"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="0.0000"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="0.000"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="0.000"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment wrapText="1" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment wrapText="1" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment wrapText="1" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment wrapText="1" readingOrder="0"/>
+    </dxf>
     <dxf>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -979,27 +1626,1015 @@
 </styleSheet>
 </file>
 
+<file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1" refreshedBy="Admin" refreshedDate="46213.488525810186" createdVersion="6" refreshedVersion="6" minRefreshableVersion="3" recordCount="24">
+  <cacheSource type="worksheet">
+    <worksheetSource name="tblGraduatePrograms"/>
+  </cacheSource>
+  <cacheFields count="17">
+    <cacheField name="University" numFmtId="0">
+      <sharedItems/>
+    </cacheField>
+    <cacheField name="Country" numFmtId="0">
+      <sharedItems count="2">
+        <s v="South Korea"/>
+        <s v="China"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="City" numFmtId="0">
+      <sharedItems/>
+    </cacheField>
+    <cacheField name="Campus study" numFmtId="0">
+      <sharedItems containsBlank="1"/>
+    </cacheField>
+    <cacheField name="Program" numFmtId="0">
+      <sharedItems/>
+    </cacheField>
+    <cacheField name="Program Category" numFmtId="0">
+      <sharedItems count="5">
+        <s v="Management Science &amp; Engineering"/>
+        <s v="Business Analytics"/>
+        <s v="Management Information Systems"/>
+        <s v="New Media Studies"/>
+        <s v="Digital Business"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="Discipline" numFmtId="0">
+      <sharedItems containsBlank="1"/>
+    </cacheField>
+    <cacheField name="Language" numFmtId="0">
+      <sharedItems containsBlank="1" count="6">
+        <s v="English / Korean"/>
+        <s v="English"/>
+        <m/>
+        <s v="Chinese"/>
+        <s v="English / Chinese"/>
+        <s v="Chinese " u="1"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="Duration (Years)" numFmtId="0">
+      <sharedItems containsString="0" containsBlank="1" containsNumber="1" minValue="2" maxValue="3"/>
+    </cacheField>
+    <cacheField name="QS Ranking " numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
+    </cacheField>
+    <cacheField name="Tuition USD" numFmtId="0">
+      <sharedItems containsString="0" containsBlank="1" containsNumber="1" minValue="8993.85" maxValue="43750" count="16">
+        <n v="8993.85"/>
+        <n v="30000"/>
+        <n v="16700"/>
+        <n v="17000"/>
+        <n v="29340"/>
+        <n v="10280"/>
+        <n v="35000"/>
+        <n v="20000"/>
+        <n v="28000"/>
+        <n v="10200"/>
+        <n v="18630"/>
+        <n v="13540"/>
+        <n v="10100"/>
+        <n v="43750"/>
+        <n v="39700"/>
+        <m/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="Scholarship Name" numFmtId="0">
+      <sharedItems containsBlank="1"/>
+    </cacheField>
+    <cacheField name="Scholarship Coverage" numFmtId="0">
+      <sharedItems containsBlank="1"/>
+    </cacheField>
+    <cacheField name="Intership Available" numFmtId="0">
+      <sharedItems containsBlank="1"/>
+    </cacheField>
+    <cacheField name="Notes" numFmtId="0">
+      <sharedItems containsBlank="1"/>
+    </cacheField>
+    <cacheField name="Data Source" numFmtId="0">
+      <sharedItems containsBlank="1"/>
+    </cacheField>
+    <cacheField name="Duplicate check" numFmtId="0">
+      <sharedItems/>
+    </cacheField>
+  </cacheFields>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
+      <x14:pivotCacheDefinition/>
+    </ext>
+  </extLst>
+</pivotCacheDefinition>
+</file>
+
+<file path=xl/pivotCache/pivotCacheRecords1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" count="24">
+  <r>
+    <s v="Korea Advanced Institute of Science and Technology (KAIST)"/>
+    <x v="0"/>
+    <s v="Daejeon"/>
+    <s v="Seoul Campus"/>
+    <s v="Management Engineering"/>
+    <x v="0"/>
+    <s v="Industrial Engineering / Operations Research"/>
+    <x v="0"/>
+    <n v="2"/>
+    <m/>
+    <x v="0"/>
+    <s v="KAIST International Student Scholarship"/>
+    <s v="Full / Partial Tuition"/>
+    <m/>
+    <s v="Scholarship awarded based on admission results. Requires verification as admission page said different"/>
+    <s v="Official KAIST Graduate School Website"/>
+    <s v="Unique"/>
+  </r>
+  <r>
+    <s v="Korea Advanced Institute of Science and Technology (KAIST)"/>
+    <x v="0"/>
+    <s v="Daejeon"/>
+    <s v="Seoul Campus"/>
+    <s v="MBA (BA tracks)"/>
+    <x v="1"/>
+    <s v="Analytics"/>
+    <x v="0"/>
+    <n v="2"/>
+    <m/>
+    <x v="1"/>
+    <s v="KAIST International Student Scholarship"/>
+    <s v="Full / Partial Tuition"/>
+    <s v="Yes"/>
+    <s v="Scholarship awarded based on admission results. Requires verification as admission page said different"/>
+    <s v="Official KAIST Graduate School Website"/>
+    <s v="Unique"/>
+  </r>
+  <r>
+    <s v="Korea University"/>
+    <x v="0"/>
+    <s v="Seoul"/>
+    <s v="Seoul Campus"/>
+    <s v="MBA (IS track)"/>
+    <x v="2"/>
+    <s v="Information Systems"/>
+    <x v="1"/>
+    <n v="2"/>
+    <m/>
+    <x v="1"/>
+    <s v="Korea International Studen Scholarship, GKS, Pony Chung, KOICA "/>
+    <s v="Full / Partial Tuition"/>
+    <m/>
+    <s v="Scholarship awarded based on admission results. Requires verification as admission page said different"/>
+    <m/>
+    <s v="Unique"/>
+  </r>
+  <r>
+    <s v="Korea University"/>
+    <x v="0"/>
+    <s v="Seoul"/>
+    <s v="Seoul Campus"/>
+    <s v="Industrial Management Engineering"/>
+    <x v="0"/>
+    <s v="Industrial Engineering / Operations Research"/>
+    <x v="0"/>
+    <n v="2"/>
+    <m/>
+    <x v="2"/>
+    <s v="Korea International Studen Scholarship, GKS, Pony Chung, KOICA "/>
+    <s v="Full / Partial Tuition"/>
+    <m/>
+    <s v="Scholarship awarded based on admission results. Requires verification as admission page said different"/>
+    <m/>
+    <s v="Unique"/>
+  </r>
+  <r>
+    <s v="Korea University"/>
+    <x v="0"/>
+    <s v="Seoul"/>
+    <s v="Seoul Campus"/>
+    <s v="Media and Communication"/>
+    <x v="3"/>
+    <s v="Media &amp; Communication"/>
+    <x v="0"/>
+    <n v="2"/>
+    <m/>
+    <x v="3"/>
+    <s v="Korea International Studen Scholarship, GKS, Pony Chung, KOICA "/>
+    <s v="Full / Partial Tuition"/>
+    <m/>
+    <s v="Scholarship awarded based on admission results. Requires verification as admission page said different"/>
+    <m/>
+    <s v="Unique"/>
+  </r>
+  <r>
+    <s v="Yonsei University"/>
+    <x v="0"/>
+    <s v="Seoul"/>
+    <s v="Seoul Campus"/>
+    <s v="MS in Information Systems (Kyobo AI and Big Data)"/>
+    <x v="2"/>
+    <m/>
+    <x v="2"/>
+    <n v="2"/>
+    <m/>
+    <x v="4"/>
+    <s v="Yonsei Global Companion Scholarship, GKS, TA/RA"/>
+    <s v="Full / Partial Tuition"/>
+    <s v="Yes"/>
+    <s v="Scholarship awarded based on admission results. "/>
+    <m/>
+    <s v="Unique"/>
+  </r>
+  <r>
+    <s v="Yonsei University"/>
+    <x v="0"/>
+    <s v="Seoul"/>
+    <s v="Seoul Campus"/>
+    <s v="MS in Information Systems, Big Data Analytics"/>
+    <x v="2"/>
+    <m/>
+    <x v="2"/>
+    <n v="2"/>
+    <m/>
+    <x v="4"/>
+    <s v="Yonsei Global Companion Scholarship, GKS, TA/RA"/>
+    <s v="Full / Partial Tuition"/>
+    <s v="Yes"/>
+    <s v="Scholarship awarded based on admission results. "/>
+    <m/>
+    <s v="Unique"/>
+  </r>
+  <r>
+    <s v="Yonsei University"/>
+    <x v="0"/>
+    <s v="Seoul"/>
+    <s v="Seoul Campus"/>
+    <s v="Digital Analytics"/>
+    <x v="1"/>
+    <s v="Analytics"/>
+    <x v="2"/>
+    <n v="2"/>
+    <m/>
+    <x v="5"/>
+    <s v="Yonsei Global Companion Scholarship, GKS, TA/RA"/>
+    <s v="Full / Partial Tuition"/>
+    <m/>
+    <s v="Scholarship awarded based on admission results. "/>
+    <m/>
+    <s v="Unique"/>
+  </r>
+  <r>
+    <s v="Yonsei University"/>
+    <x v="0"/>
+    <s v="Seoul"/>
+    <s v="Seoul Campus"/>
+    <s v="Global MBA"/>
+    <x v="4"/>
+    <s v="Busienss &amp; Technology"/>
+    <x v="0"/>
+    <n v="2"/>
+    <m/>
+    <x v="6"/>
+    <s v="University Scholarship, GKS"/>
+    <s v="Full / Partial Tuition"/>
+    <s v="Yes"/>
+    <s v="Scholarship awarded based on admission results and need tp re-apply each semester. "/>
+    <m/>
+    <s v="Unique"/>
+  </r>
+  <r>
+    <s v="Yonsei University"/>
+    <x v="0"/>
+    <s v="Seoul"/>
+    <s v="Seoul Campus"/>
+    <s v="Media and Communication"/>
+    <x v="3"/>
+    <s v="Media &amp; Communication"/>
+    <x v="0"/>
+    <m/>
+    <m/>
+    <x v="7"/>
+    <s v="University Scholarship, GKS"/>
+    <s v="Full / Partial Tuition"/>
+    <m/>
+    <s v="Scholarship awarded based on admission results and need tp re-apply each semester. "/>
+    <m/>
+    <s v="Unique"/>
+  </r>
+  <r>
+    <s v="Hanyang University"/>
+    <x v="0"/>
+    <s v="Seoul"/>
+    <s v="Seoul Campus"/>
+    <s v="Industrial Engineering (DA Track)"/>
+    <x v="1"/>
+    <s v="Analytics"/>
+    <x v="0"/>
+    <n v="2"/>
+    <m/>
+    <x v="7"/>
+    <s v="Hanyang International Scholarship Program (HISP), Assistantships, Language Proficiency "/>
+    <s v="Full / Partial Tuition"/>
+    <m/>
+    <m/>
+    <m/>
+    <s v="Unique"/>
+  </r>
+  <r>
+    <s v="Hanyang University"/>
+    <x v="0"/>
+    <s v="Seoul"/>
+    <s v="Erica Campus"/>
+    <s v="Media and Social Informatics "/>
+    <x v="3"/>
+    <s v="Media &amp; Communication"/>
+    <x v="0"/>
+    <n v="2"/>
+    <m/>
+    <x v="8"/>
+    <s v="Hanyang International Scholarship Program (HISP), Assistantships, Language Proficiency "/>
+    <s v="Full / Partial Tuition"/>
+    <m/>
+    <m/>
+    <m/>
+    <s v="Unique"/>
+  </r>
+  <r>
+    <s v="Kyunghee University "/>
+    <x v="0"/>
+    <s v="Seoul"/>
+    <s v="Seoul Campus"/>
+    <s v="Journalism &amp; Communication"/>
+    <x v="3"/>
+    <s v="Media &amp; Communication"/>
+    <x v="0"/>
+    <n v="2"/>
+    <m/>
+    <x v="9"/>
+    <s v="President's Scholarship, Merit Maintanance "/>
+    <s v="Full / Partial Tuition"/>
+    <m/>
+    <m/>
+    <m/>
+    <s v="Unique"/>
+  </r>
+  <r>
+    <s v="Ewha Women University"/>
+    <x v="0"/>
+    <s v="Seoul"/>
+    <m/>
+    <s v="Media and Communication"/>
+    <x v="3"/>
+    <s v="Media &amp; Communication"/>
+    <x v="0"/>
+    <n v="2"/>
+    <m/>
+    <x v="9"/>
+    <s v="Ehwa University Scholarship, Ewha Research Excellence, Outstanding Ewha Science Student"/>
+    <s v="Full / Partial Tuition"/>
+    <m/>
+    <s v="Scholarship awarded based on admission results and need tp re-apply each semester. "/>
+    <m/>
+    <s v="Unique"/>
+  </r>
+  <r>
+    <s v="Ewha Women University"/>
+    <x v="0"/>
+    <s v="Seoul"/>
+    <m/>
+    <s v="Big Data Analytics"/>
+    <x v="1"/>
+    <s v="Analytics"/>
+    <x v="0"/>
+    <n v="2"/>
+    <m/>
+    <x v="10"/>
+    <s v="Ehwa University Scholarship, Ewha Research Excellence, Outstanding Ewha Science Student"/>
+    <s v="Full / Partial Tuition"/>
+    <m/>
+    <s v="Scholarship awarded based on admission results and need tp re-apply each semester. "/>
+    <m/>
+    <s v="Unique"/>
+  </r>
+  <r>
+    <s v="Ewha Women University"/>
+    <x v="0"/>
+    <s v="Seoul"/>
+    <m/>
+    <s v="Big Data MBA (BA track)"/>
+    <x v="1"/>
+    <s v="Analytics"/>
+    <x v="0"/>
+    <n v="2"/>
+    <m/>
+    <x v="1"/>
+    <s v="Ehwa University Scholarship, Ewha Research Excellence, Outstanding Ewha Science Student"/>
+    <s v="Full / Partial Tuition"/>
+    <m/>
+    <s v="Scholarship awarded based on admission results and need tp re-apply each semester. "/>
+    <m/>
+    <s v="Unique"/>
+  </r>
+  <r>
+    <s v="Zhejiang University"/>
+    <x v="1"/>
+    <s v="Hangzhou"/>
+    <m/>
+    <s v="MSE"/>
+    <x v="0"/>
+    <s v="Management &amp; Engineering"/>
+    <x v="1"/>
+    <n v="2.5"/>
+    <m/>
+    <x v="11"/>
+    <s v="Chinese Government Scholarship (CGS), Zhejiang University Scholarship, Zhejiang Government Scholarship "/>
+    <s v="Full / Partial Tuition + Living Stipend"/>
+    <m/>
+    <m/>
+    <m/>
+    <s v="Unique"/>
+  </r>
+  <r>
+    <s v="Zhejiang University"/>
+    <x v="1"/>
+    <s v="Hangzhou"/>
+    <m/>
+    <s v="Communication"/>
+    <x v="2"/>
+    <s v="Media &amp; Communication"/>
+    <x v="3"/>
+    <n v="3"/>
+    <m/>
+    <x v="12"/>
+    <s v="Chinese Government Scholarship (CGS), Zhejiang University Scholarship, Zhejiang Government Scholarship "/>
+    <s v="Full / Partial Tuition + Living Stipend"/>
+    <m/>
+    <m/>
+    <m/>
+    <s v="Unique"/>
+  </r>
+  <r>
+    <s v="Zhejiang University"/>
+    <x v="1"/>
+    <s v="Hangzhou"/>
+    <m/>
+    <s v="Information and Communication Engineering"/>
+    <x v="2"/>
+    <s v="Information Systems"/>
+    <x v="3"/>
+    <n v="3"/>
+    <m/>
+    <x v="12"/>
+    <s v="Chinese Government Scholarship (CGS), Zhejiang University Scholarship, Zhejiang Government Scholarship "/>
+    <s v="Full / Partial Tuition + Living Stipend"/>
+    <m/>
+    <m/>
+    <m/>
+    <s v="Unique"/>
+  </r>
+  <r>
+    <s v="Shanghai Jiaotong University"/>
+    <x v="1"/>
+    <s v="Shanghai"/>
+    <s v="Antai College"/>
+    <s v="MSE"/>
+    <x v="0"/>
+    <s v="Management &amp; Engineering"/>
+    <x v="4"/>
+    <n v="2.5"/>
+    <m/>
+    <x v="13"/>
+    <s v="Chinese Government Scholarship (CGS), Antai College Specific Scholarships, Shanghai Government Scholarship "/>
+    <s v="Full / Partial Tuition_x000a_"/>
+    <m/>
+    <m/>
+    <m/>
+    <s v="Unique"/>
+  </r>
+  <r>
+    <s v="Fudan University"/>
+    <x v="1"/>
+    <s v="Shanghai"/>
+    <m/>
+    <s v="Data Science and Business Analytics (DS&amp;BA)"/>
+    <x v="1"/>
+    <s v="Analytics"/>
+    <x v="4"/>
+    <n v="2"/>
+    <m/>
+    <x v="14"/>
+    <s v="Xing Quan Belt and Road Scholarship,  Chinese Government Scholarship"/>
+    <s v="Full / Partial Tuition_x000a_"/>
+    <m/>
+    <m/>
+    <m/>
+    <s v="Unique"/>
+  </r>
+  <r>
+    <s v="Renmin University of China "/>
+    <x v="1"/>
+    <s v="Beijing"/>
+    <m/>
+    <s v="Information Management"/>
+    <x v="2"/>
+    <s v="Information Systems"/>
+    <x v="4"/>
+    <n v="2"/>
+    <m/>
+    <x v="15"/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <s v="Unique"/>
+  </r>
+  <r>
+    <s v="Communication University of China (CUC)"/>
+    <x v="1"/>
+    <s v="Beijing"/>
+    <m/>
+    <s v="New Media studies"/>
+    <x v="3"/>
+    <s v="Media &amp; Communication"/>
+    <x v="4"/>
+    <n v="2"/>
+    <m/>
+    <x v="15"/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <s v="Unique"/>
+  </r>
+  <r>
+    <s v="Shanghai Jiaotong University"/>
+    <x v="1"/>
+    <s v="Shanghai"/>
+    <m/>
+    <s v="New Media studies"/>
+    <x v="3"/>
+    <s v="Media &amp; Communication"/>
+    <x v="1"/>
+    <n v="2"/>
+    <m/>
+    <x v="12"/>
+    <s v="Chinese Government Scholarship (CGS), Antai College Specific Scholarships, Shanghai Government Scholarship "/>
+    <s v="Full / Partial Tuition_x000a_"/>
+    <m/>
+    <m/>
+    <m/>
+    <s v="Unique"/>
+  </r>
+</pivotCacheRecords>
+</file>
+
+<file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="ptAverageTuition" cacheId="10" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
+  <location ref="A35:B38" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="17">
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField axis="axisRow" compact="0" outline="0" showAll="0">
+      <items count="3">
+        <item x="1"/>
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0">
+      <items count="7">
+        <item x="3"/>
+        <item m="1" x="5"/>
+        <item x="1"/>
+        <item x="4"/>
+        <item x="0"/>
+        <item x="2"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField dataField="1" compact="0" outline="0" showAll="0">
+      <items count="17">
+        <item x="0"/>
+        <item x="12"/>
+        <item x="9"/>
+        <item x="5"/>
+        <item x="11"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="10"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item x="4"/>
+        <item x="1"/>
+        <item x="6"/>
+        <item x="14"/>
+        <item x="13"/>
+        <item x="15"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="1"/>
+  </rowFields>
+  <rowItems count="3">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Average of Tuition USD" fld="10" subtotal="average" baseField="1" baseItem="0" numFmtId="2"/>
+  </dataFields>
+  <formats count="16">
+    <format dxfId="173">
+      <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="174">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+    <format dxfId="175">
+      <pivotArea field="7" type="button" dataOnly="0" labelOnly="1" outline="0"/>
+    </format>
+    <format dxfId="176">
+      <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
+    </format>
+    <format dxfId="177">
+      <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="178">
+      <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
+    </format>
+    <format dxfId="108">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+    <format dxfId="100">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+    <format dxfId="91">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+    <format dxfId="81">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+    <format dxfId="70">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+    <format dxfId="58">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+    <format dxfId="45">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+    <format dxfId="31">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+    <format dxfId="16">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+    <format dxfId="0">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+  </formats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="ptLanguage" cacheId="10" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
+  <location ref="A23:B29" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="17">
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField dataField="1" compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField axis="axisRow" compact="0" outline="0" showAll="0">
+      <items count="7">
+        <item x="3"/>
+        <item m="1" x="5"/>
+        <item x="1"/>
+        <item x="4"/>
+        <item x="0"/>
+        <item x="2"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="7"/>
+  </rowFields>
+  <rowItems count="6">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i>
+      <x v="5"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Count of Program" fld="4" subtotal="count" baseField="0" baseItem="0"/>
+  </dataFields>
+  <formats count="8">
+    <format dxfId="201">
+      <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="7" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="199">
+      <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="198">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+    <format dxfId="197">
+      <pivotArea field="7" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
+    </format>
+    <format dxfId="196">
+      <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
+    </format>
+    <format dxfId="195">
+      <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="7" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="194">
+      <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="193">
+      <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
+    </format>
+  </formats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="ptProgramCategory" cacheId="10" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
+  <location ref="A11:B17" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="17">
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField dataField="1" compact="0" outline="0" showAll="0"/>
+    <pivotField axis="axisRow" compact="0" outline="0" showAll="0">
+      <items count="6">
+        <item x="1"/>
+        <item x="4"/>
+        <item x="2"/>
+        <item x="0"/>
+        <item x="3"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="5"/>
+  </rowFields>
+  <rowItems count="6">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Count of Program" fld="4" subtotal="count" baseField="0" baseItem="0"/>
+  </dataFields>
+  <formats count="8">
+    <format dxfId="200">
+      <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="5" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="192">
+      <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="191">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+    <format dxfId="190">
+      <pivotArea field="5" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
+    </format>
+    <format dxfId="189">
+      <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
+    </format>
+    <format dxfId="188">
+      <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="5" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="187">
+      <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="186">
+      <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
+    </format>
+  </formats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="ptCountry" cacheId="10" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
+  <location ref="A2:B5" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="17">
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField axis="axisRow" compact="0" outline="0" showAll="0">
+      <items count="3">
+        <item x="1"/>
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField dataField="1" compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="1"/>
+  </rowFields>
+  <rowItems count="3">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Count of Program" fld="4" subtotal="count" baseField="0" baseItem="0"/>
+  </dataFields>
+  <formats count="7">
+    <format dxfId="185">
+      <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="184">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+    <format dxfId="183">
+      <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
+    </format>
+    <format dxfId="182">
+      <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
+    </format>
+    <format dxfId="181">
+      <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="1" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="180">
+      <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="179">
+      <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
+    </format>
+  </formats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="tblGraduatePrograms" displayName="tblGraduatePrograms" ref="A1:Q25" totalsRowShown="0" dataDxfId="17" headerRowCellStyle="Normal" dataCellStyle="Normal">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="tblGraduatePrograms" displayName="tblGraduatePrograms" ref="A1:Q25" totalsRowShown="0" dataDxfId="219" headerRowCellStyle="Normal" dataCellStyle="Normal">
   <autoFilter ref="A1:Q25"/>
   <tableColumns count="17">
-    <tableColumn id="1" name="University" dataDxfId="16" dataCellStyle="Normal"/>
-    <tableColumn id="2" name="Country" dataDxfId="15" dataCellStyle="Normal"/>
-    <tableColumn id="3" name="City" dataDxfId="14" dataCellStyle="Normal"/>
-    <tableColumn id="16" name="Campus study" dataDxfId="13"/>
-    <tableColumn id="4" name="Program" dataDxfId="12" dataCellStyle="Normal"/>
-    <tableColumn id="5" name="Program Category" dataDxfId="11" dataCellStyle="Normal"/>
-    <tableColumn id="6" name="Discipline" dataDxfId="10" dataCellStyle="Normal"/>
-    <tableColumn id="7" name="Language" dataDxfId="9" dataCellStyle="Normal"/>
-    <tableColumn id="8" name="Duration (Years)" dataDxfId="8" dataCellStyle="Normal"/>
-    <tableColumn id="9" name="QS Ranking " dataDxfId="7" dataCellStyle="Normal"/>
-    <tableColumn id="10" name="Tuition USD" dataDxfId="6" dataCellStyle="Normal"/>
-    <tableColumn id="11" name="Scholarship Name" dataDxfId="5" dataCellStyle="Normal"/>
-    <tableColumn id="12" name="Scholarship Coverage" dataDxfId="4" dataCellStyle="Normal"/>
-    <tableColumn id="13" name="Intership Available" dataDxfId="3" dataCellStyle="Normal"/>
-    <tableColumn id="15" name="Notes" dataDxfId="2"/>
-    <tableColumn id="17" name="Data Source" dataDxfId="1"/>
-    <tableColumn id="14" name="Duplicate check" dataDxfId="0" dataCellStyle="Normal">
+    <tableColumn id="1" name="University" dataDxfId="218" dataCellStyle="Normal"/>
+    <tableColumn id="2" name="Country" dataDxfId="217" dataCellStyle="Normal"/>
+    <tableColumn id="3" name="City" dataDxfId="216" dataCellStyle="Normal"/>
+    <tableColumn id="16" name="Campus study" dataDxfId="215"/>
+    <tableColumn id="4" name="Program" dataDxfId="214" dataCellStyle="Normal"/>
+    <tableColumn id="5" name="Program Category" dataDxfId="213" dataCellStyle="Normal"/>
+    <tableColumn id="6" name="Discipline" dataDxfId="212" dataCellStyle="Normal"/>
+    <tableColumn id="7" name="Language" dataDxfId="211" dataCellStyle="Normal"/>
+    <tableColumn id="8" name="Duration (Years)" dataDxfId="210" dataCellStyle="Normal"/>
+    <tableColumn id="9" name="QS Ranking " dataDxfId="209" dataCellStyle="Normal"/>
+    <tableColumn id="10" name="Tuition USD" dataDxfId="208" dataCellStyle="Normal"/>
+    <tableColumn id="11" name="Scholarship Name" dataDxfId="207" dataCellStyle="Normal"/>
+    <tableColumn id="12" name="Scholarship Coverage" dataDxfId="206" dataCellStyle="Normal"/>
+    <tableColumn id="13" name="Intership Available" dataDxfId="205" dataCellStyle="Normal"/>
+    <tableColumn id="15" name="Notes" dataDxfId="204"/>
+    <tableColumn id="17" name="Data Source" dataDxfId="203"/>
+    <tableColumn id="14" name="Duplicate check" dataDxfId="202" dataCellStyle="Normal">
       <calculatedColumnFormula>IF(COUNTIFS(tblGraduatePrograms[University],tblGraduatePrograms[[#This Row],[University]],tblGraduatePrograms[Program],tblGraduatePrograms[[#This Row],[Program]])&gt;1,"Duplicate","Unique")</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1365,7 +3000,7 @@
         <v>8</v>
       </c>
       <c r="N1" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="O1" t="s">
         <v>9</v>
@@ -1374,7 +3009,7 @@
         <v>143</v>
       </c>
       <c r="Q1" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
     </row>
     <row r="2" spans="1:17" ht="114" customHeight="1" x14ac:dyDescent="0.25">
@@ -1417,7 +3052,7 @@
       </c>
       <c r="N2" s="12"/>
       <c r="O2" s="12" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="P2" s="12" t="s">
         <v>149</v>
@@ -1469,7 +3104,7 @@
         <v>79</v>
       </c>
       <c r="O3" s="12" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="P3" s="12" t="s">
         <v>149</v>
@@ -1496,7 +3131,7 @@
         <v>155</v>
       </c>
       <c r="F4" s="12" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="G4" s="12" t="s">
         <v>34</v>
@@ -1519,7 +3154,7 @@
       </c>
       <c r="N4" s="13"/>
       <c r="O4" s="12" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="P4" s="12"/>
       <c r="Q4" s="12" t="str">
@@ -1567,7 +3202,7 @@
       </c>
       <c r="N5" s="13"/>
       <c r="O5" s="12" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="P5" s="13"/>
       <c r="Q5" s="12" t="str">
@@ -1592,7 +3227,7 @@
         <v>158</v>
       </c>
       <c r="F6" s="12" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="G6" s="12" t="s">
         <v>37</v>
@@ -1615,7 +3250,7 @@
       </c>
       <c r="N6" s="13"/>
       <c r="O6" s="12" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="P6" s="12"/>
       <c r="Q6" s="12" t="str">
@@ -1640,7 +3275,7 @@
         <v>172</v>
       </c>
       <c r="F7" s="12" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="G7" s="13"/>
       <c r="H7" s="13"/>
@@ -1686,7 +3321,7 @@
         <v>171</v>
       </c>
       <c r="F8" s="12" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="G8" s="13"/>
       <c r="H8" s="13"/>
@@ -1778,7 +3413,7 @@
         <v>161</v>
       </c>
       <c r="F10" s="12" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="G10" s="12" t="s">
         <v>35</v>
@@ -1828,7 +3463,7 @@
         <v>158</v>
       </c>
       <c r="F11" s="12" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="G11" s="12" t="s">
         <v>37</v>
@@ -1920,7 +3555,7 @@
         <v>167</v>
       </c>
       <c r="F13" s="12" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="G13" s="12" t="s">
         <v>37</v>
@@ -1963,10 +3598,10 @@
         <v>151</v>
       </c>
       <c r="E14" s="13" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="F14" s="12" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="G14" s="12" t="s">
         <v>37</v>
@@ -1982,7 +3617,7 @@
         <v>10200</v>
       </c>
       <c r="L14" s="13" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="M14" s="12" t="s">
         <v>154</v>
@@ -2010,7 +3645,7 @@
         <v>158</v>
       </c>
       <c r="F15" s="12" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="G15" s="12" t="s">
         <v>37</v>
@@ -2167,7 +3802,7 @@
         <v>174</v>
       </c>
       <c r="M18" s="12" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="N18" s="12"/>
       <c r="O18" s="12"/>
@@ -2192,13 +3827,13 @@
         <v>175</v>
       </c>
       <c r="F19" s="12" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="G19" s="12" t="s">
         <v>37</v>
       </c>
       <c r="H19" s="13" t="s">
-        <v>176</v>
+        <v>200</v>
       </c>
       <c r="I19" s="13">
         <v>3</v>
@@ -2211,7 +3846,7 @@
         <v>174</v>
       </c>
       <c r="M19" s="12" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="N19" s="13"/>
       <c r="O19" s="12"/>
@@ -2233,16 +3868,16 @@
       </c>
       <c r="D20" s="12"/>
       <c r="E20" s="13" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="F20" s="12" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="G20" s="12" t="s">
         <v>34</v>
       </c>
       <c r="H20" s="13" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="I20" s="13">
         <v>3</v>
@@ -2255,7 +3890,7 @@
         <v>174</v>
       </c>
       <c r="M20" s="12" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="N20" s="13"/>
       <c r="O20" s="12"/>
@@ -2276,7 +3911,7 @@
         <v>30</v>
       </c>
       <c r="D21" s="12" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="E21" s="12" t="s">
         <v>27</v>
@@ -2288,7 +3923,7 @@
         <v>33</v>
       </c>
       <c r="H21" s="12" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="I21" s="12">
         <v>2.5</v>
@@ -2298,10 +3933,10 @@
         <v>43750</v>
       </c>
       <c r="L21" s="12" t="s">
+        <v>178</v>
+      </c>
+      <c r="M21" s="12" t="s">
         <v>179</v>
-      </c>
-      <c r="M21" s="12" t="s">
-        <v>180</v>
       </c>
       <c r="N21" s="12"/>
       <c r="O21" s="12"/>
@@ -2323,7 +3958,7 @@
       </c>
       <c r="D22" s="12"/>
       <c r="E22" s="12" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="F22" s="12" t="s">
         <v>17</v>
@@ -2332,7 +3967,7 @@
         <v>36</v>
       </c>
       <c r="H22" s="12" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="I22" s="12">
         <v>2</v>
@@ -2342,10 +3977,10 @@
         <v>39700</v>
       </c>
       <c r="L22" s="12" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="M22" s="12" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="N22" s="12"/>
       <c r="O22" s="12"/>
@@ -2370,13 +4005,13 @@
         <v>32</v>
       </c>
       <c r="F23" s="12" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="G23" s="12" t="s">
         <v>34</v>
       </c>
       <c r="H23" s="12" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="I23" s="12">
         <v>2</v>
@@ -2408,13 +4043,13 @@
         <v>28</v>
       </c>
       <c r="F24" s="12" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="G24" s="12" t="s">
         <v>37</v>
       </c>
       <c r="H24" s="12" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="I24" s="12">
         <v>2</v>
@@ -2446,7 +4081,7 @@
         <v>28</v>
       </c>
       <c r="F25" s="12" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="G25" s="12" t="s">
         <v>37</v>
@@ -2462,10 +4097,10 @@
         <v>10100</v>
       </c>
       <c r="L25" s="12" t="s">
+        <v>178</v>
+      </c>
+      <c r="M25" s="12" t="s">
         <v>179</v>
-      </c>
-      <c r="M25" s="12" t="s">
-        <v>180</v>
       </c>
       <c r="N25" s="12"/>
       <c r="O25" s="12"/>
@@ -2522,28 +4157,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" s="23" t="s">
+      <c r="A1" s="16" t="s">
+        <v>216</v>
+      </c>
+      <c r="B1" s="16" t="s">
         <v>217</v>
       </c>
-      <c r="B1" s="23" t="s">
+      <c r="C1" s="18" t="s">
         <v>218</v>
       </c>
-      <c r="C1" s="25" t="s">
-        <v>219</v>
-      </c>
-      <c r="D1" s="23" t="s">
-        <v>215</v>
+      <c r="D1" s="16" t="s">
+        <v>214</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="12" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="B2" s="12">
         <f>COUNTA(tblGraduatePrograms[Program])</f>
         <v>24</v>
       </c>
-      <c r="C2" s="24"/>
+      <c r="C2" s="17"/>
       <c r="D2" s="12" t="str">
         <f>"✅ Updated"</f>
         <v>✅ Updated</v>
@@ -2551,13 +4186,13 @@
     </row>
     <row r="3" spans="1:4" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="12" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B3" s="12">
         <f>COUNTIF(tblGraduatePrograms[Duplicate check],"Duplicate")</f>
         <v>0</v>
       </c>
-      <c r="C3" s="24"/>
+      <c r="C3" s="17"/>
       <c r="D3" s="12" t="str">
         <f>IF(B3=0,"🟢 Excellent","🔴 Duplicate Found")</f>
         <v>🟢 Excellent</v>
@@ -2565,13 +4200,13 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="B4" s="12">
         <f>COUNTBLANK(tblGraduatePrograms[Tuition USD])</f>
         <v>2</v>
       </c>
-      <c r="C4" s="24"/>
+      <c r="C4" s="17"/>
       <c r="D4" s="12" t="str">
         <f>IF(B4=0,"🟢 Complete","🟡 Need Update")</f>
         <v>🟡 Need Update</v>
@@ -2579,13 +4214,13 @@
     </row>
     <row r="5" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="12" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B5" s="12">
         <f>COUNTBLANK(tblGraduatePrograms[Scholarship Name])</f>
         <v>2</v>
       </c>
-      <c r="C5" s="24"/>
+      <c r="C5" s="17"/>
       <c r="D5" s="12" t="str">
         <f>IF(B5=0,"🟢 Complete","🟡 Need Update")</f>
         <v>🟡 Need Update</v>
@@ -2593,27 +4228,27 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="12" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="B6" s="12">
         <f>COUNTBLANK(tblGraduatePrograms[Language])</f>
         <v>3</v>
       </c>
-      <c r="C6" s="24"/>
+      <c r="C6" s="17"/>
       <c r="D6" s="12" t="str">
         <f>IF(B6=0,"🟢 Complete","🟡 Need Update")</f>
         <v>🟡 Need Update</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="12" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="B7" s="12">
         <f>COUNTBLANK(tblGraduatePrograms[Intership Available])</f>
         <v>20</v>
       </c>
-      <c r="C7" s="24"/>
+      <c r="C7" s="17"/>
       <c r="D7" s="12" t="str">
         <f>IF(B7=0,"🟢 Complete","🟡 Need Verification")</f>
         <v>🟡 Need Verification</v>
@@ -2621,13 +4256,13 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="12" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="B8" s="12">
         <f>COUNTBLANK(tblGraduatePrograms[[QS Ranking ]])</f>
         <v>24</v>
       </c>
-      <c r="C8" s="24"/>
+      <c r="C8" s="17"/>
       <c r="D8" s="12" t="str">
         <f>IF(B8=0,"🟢 Complete","🟡 Need Update")</f>
         <v>🟡 Need Update</v>
@@ -2635,13 +4270,13 @@
     </row>
     <row r="9" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="12" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="B9" s="12">
         <f>COUNTIF(tblGraduatePrograms[Country],"South Korea")</f>
         <v>16</v>
       </c>
-      <c r="C9" s="24"/>
+      <c r="C9" s="17"/>
       <c r="D9" s="12" t="str">
         <f>"✅ OK"</f>
         <v>✅ OK</v>
@@ -2649,13 +4284,13 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="12" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="B10" s="12">
         <f>COUNTIF(tblGraduatePrograms[Country],"China")</f>
         <v>8</v>
       </c>
-      <c r="C10" s="24"/>
+      <c r="C10" s="17"/>
       <c r="D10" s="12" t="str">
         <f>"✅ OK"</f>
         <v>✅ OK</v>
@@ -2663,13 +4298,13 @@
     </row>
     <row r="11" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A11" s="12" t="s">
-        <v>229</v>
-      </c>
-      <c r="B11" s="26">
+        <v>228</v>
+      </c>
+      <c r="B11" s="19">
         <f>AVERAGE(tblGraduatePrograms[Tuition USD])</f>
         <v>21407.902272727271</v>
       </c>
-      <c r="C11" s="24"/>
+      <c r="C11" s="17"/>
       <c r="D11" s="12" t="str">
         <f>"📊 Calculated"</f>
         <v>📊 Calculated</v>
@@ -2677,13 +4312,13 @@
     </row>
     <row r="12" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" s="12" t="s">
-        <v>230</v>
-      </c>
-      <c r="B12" s="26">
+        <v>229</v>
+      </c>
+      <c r="B12" s="19">
         <f>MAX(tblGraduatePrograms[Tuition USD])</f>
         <v>43750</v>
       </c>
-      <c r="C12" s="24"/>
+      <c r="C12" s="17"/>
       <c r="D12" s="12" t="str">
         <f>"📊 Calculated"</f>
         <v>📊 Calculated</v>
@@ -2691,13 +4326,13 @@
     </row>
     <row r="13" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A13" s="12" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="B13" s="12">
         <f>MIN(tblGraduatePrograms[Tuition USD])</f>
         <v>8993.85</v>
       </c>
-      <c r="C13" s="24"/>
+      <c r="C13" s="17"/>
       <c r="D13" s="12" t="str">
         <f>"📊 Calculated"</f>
         <v>📊 Calculated</v>
@@ -2723,39 +4358,39 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="22" t="s">
         <v>25</v>
       </c>
-      <c r="B1" s="18"/>
+      <c r="B1" s="22"/>
       <c r="C1" s="12"/>
-      <c r="D1" s="18" t="s">
-        <v>191</v>
-      </c>
-      <c r="E1" s="18"/>
+      <c r="D1" s="22" t="s">
+        <v>190</v>
+      </c>
+      <c r="E1" s="22"/>
       <c r="F1" s="12"/>
-      <c r="G1" s="18" t="s">
+      <c r="G1" s="22" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="18"/>
+      <c r="H1" s="22"/>
       <c r="I1" s="12"/>
-      <c r="J1" s="18" t="s">
+      <c r="J1" s="22" t="s">
         <v>1</v>
       </c>
-      <c r="K1" s="18"/>
+      <c r="K1" s="22"/>
       <c r="L1" s="15"/>
-      <c r="M1" s="16" t="s">
+      <c r="M1" s="20" t="s">
         <v>8</v>
       </c>
-      <c r="N1" s="16"/>
+      <c r="N1" s="20"/>
       <c r="O1" s="15"/>
-      <c r="P1" s="16" t="s">
-        <v>208</v>
-      </c>
-      <c r="Q1" s="16"/>
-      <c r="S1" s="17" t="s">
-        <v>210</v>
-      </c>
-      <c r="T1" s="17"/>
+      <c r="P1" s="20" t="s">
+        <v>207</v>
+      </c>
+      <c r="Q1" s="20"/>
+      <c r="S1" s="21" t="s">
+        <v>209</v>
+      </c>
+      <c r="T1" s="21"/>
     </row>
     <row r="2" spans="1:20" ht="45" x14ac:dyDescent="0.25">
       <c r="A2" s="12" t="s">
@@ -2779,7 +4414,7 @@
       <c r="K2" s="12"/>
       <c r="L2" s="15"/>
       <c r="M2" s="15" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="N2" s="15"/>
       <c r="O2" s="15"/>
@@ -2788,7 +4423,7 @@
       </c>
       <c r="Q2" s="15"/>
       <c r="S2" s="6" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="3" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2803,7 +4438,7 @@
       <c r="E3" s="12"/>
       <c r="F3" s="12"/>
       <c r="G3" s="12" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="H3" s="12"/>
       <c r="I3" s="12"/>
@@ -2813,31 +4448,31 @@
       <c r="K3" s="12"/>
       <c r="L3" s="15"/>
       <c r="M3" s="15" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="N3" s="15"/>
       <c r="O3" s="15"/>
       <c r="P3" s="15" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="Q3" s="15"/>
       <c r="S3" s="6" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="4" spans="1:20" ht="45" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="B4" s="12"/>
       <c r="C4" s="12"/>
       <c r="D4" s="12" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="E4" s="12"/>
       <c r="F4" s="12"/>
       <c r="G4" s="12" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="H4" s="12"/>
       <c r="I4" s="12"/>
@@ -2852,17 +4487,17 @@
       <c r="P4" s="15"/>
       <c r="Q4" s="15"/>
       <c r="S4" s="3" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="5" spans="1:20" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="12" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B5" s="12"/>
       <c r="C5" s="12"/>
       <c r="D5" s="12" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="E5" s="12"/>
       <c r="F5" s="12"/>
@@ -2875,19 +4510,19 @@
       <c r="K5" s="12"/>
       <c r="L5" s="15"/>
       <c r="M5" s="15" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="N5" s="15"/>
       <c r="O5" s="15"/>
       <c r="P5" s="15"/>
       <c r="Q5" s="15"/>
       <c r="S5" s="3" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="6" spans="1:20" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="12" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="B6" s="12"/>
       <c r="C6" s="12"/>
@@ -2897,7 +4532,7 @@
       <c r="E6" s="12"/>
       <c r="F6" s="12"/>
       <c r="G6" s="12" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="H6" s="12"/>
       <c r="I6" s="12"/>
@@ -2905,29 +4540,29 @@
       <c r="K6" s="12"/>
       <c r="L6" s="15"/>
       <c r="M6" s="15" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="N6" s="15"/>
       <c r="O6" s="15"/>
       <c r="P6" s="15"/>
       <c r="Q6" s="15"/>
       <c r="S6" s="6" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="7" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A7" s="12" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B7" s="12"/>
       <c r="C7" s="12"/>
       <c r="D7" s="12" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="E7" s="12"/>
       <c r="F7" s="12"/>
       <c r="G7" s="12" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="H7" s="12"/>
       <c r="I7" s="12"/>
@@ -2943,17 +4578,17 @@
     </row>
     <row r="8" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A8" s="12" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B8" s="12"/>
       <c r="C8" s="12"/>
       <c r="D8" s="12" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="E8" s="12"/>
       <c r="F8" s="12"/>
       <c r="G8" s="12" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="H8" s="12"/>
       <c r="I8" s="12"/>
@@ -2972,7 +4607,7 @@
       <c r="B9" s="15"/>
       <c r="C9" s="15"/>
       <c r="D9" s="15" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="E9" s="15"/>
       <c r="F9" s="15"/>
@@ -2994,7 +4629,7 @@
       <c r="B10" s="15"/>
       <c r="C10" s="15"/>
       <c r="D10" s="12" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="E10" s="15"/>
       <c r="F10" s="15"/>
@@ -3373,26 +5008,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="24" t="s">
         <v>108</v>
       </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20"/>
-      <c r="D1" s="20"/>
-      <c r="E1" s="20"/>
-      <c r="F1" s="20"/>
-      <c r="G1" s="20"/>
-      <c r="H1" s="20"/>
+      <c r="B1" s="24"/>
+      <c r="C1" s="24"/>
+      <c r="D1" s="24"/>
+      <c r="E1" s="24"/>
+      <c r="F1" s="24"/>
+      <c r="G1" s="24"/>
+      <c r="H1" s="24"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="10"/>
       <c r="B2" s="10"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A3" s="21" t="s">
+      <c r="A3" s="25" t="s">
         <v>134</v>
       </c>
-      <c r="B3" s="21"/>
+      <c r="B3" s="25"/>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
@@ -3451,22 +5086,22 @@
       </c>
     </row>
     <row r="13" spans="1:8" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="18" t="s">
+      <c r="A13" s="22" t="s">
         <v>123</v>
       </c>
-      <c r="B13" s="18"/>
-      <c r="C13" s="18"/>
-      <c r="D13" s="18"/>
-      <c r="E13" s="18"/>
-      <c r="F13" s="18"/>
-      <c r="G13" s="18"/>
-      <c r="H13" s="18"/>
+      <c r="B13" s="22"/>
+      <c r="C13" s="22"/>
+      <c r="D13" s="22"/>
+      <c r="E13" s="22"/>
+      <c r="F13" s="22"/>
+      <c r="G13" s="22"/>
+      <c r="H13" s="22"/>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A18" s="22" t="s">
+      <c r="A18" s="26" t="s">
         <v>135</v>
       </c>
-      <c r="B18" s="22"/>
+      <c r="B18" s="26"/>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
@@ -3517,10 +5152,10 @@
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A28" s="22" t="s">
+      <c r="A28" s="26" t="s">
         <v>136</v>
       </c>
-      <c r="B28" s="22"/>
+      <c r="B28" s="26"/>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
@@ -3555,10 +5190,10 @@
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A36" s="22" t="s">
+      <c r="A36" s="26" t="s">
         <v>137</v>
       </c>
-      <c r="B36" s="22"/>
+      <c r="B36" s="26"/>
     </row>
     <row r="37" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
@@ -3597,10 +5232,10 @@
       <c r="C40" s="10"/>
     </row>
     <row r="45" spans="1:3" ht="18" x14ac:dyDescent="0.25">
-      <c r="A45" s="19" t="s">
+      <c r="A45" s="23" t="s">
         <v>138</v>
       </c>
-      <c r="B45" s="19"/>
+      <c r="B45" s="23"/>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
@@ -3637,4 +5272,249 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:B38"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="18.140625" customWidth="1"/>
+    <col min="2" max="2" width="21.85546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A1" s="30" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" s="27" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="15" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" s="15" t="s">
+        <v>26</v>
+      </c>
+      <c r="B3" s="28">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" s="15" t="s">
+        <v>14</v>
+      </c>
+      <c r="B4" s="28">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" s="15" t="s">
+        <v>232</v>
+      </c>
+      <c r="B5" s="28">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" s="15"/>
+      <c r="B6" s="15"/>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" s="15"/>
+      <c r="B7" s="15"/>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" s="15"/>
+      <c r="B8" s="15"/>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" s="15"/>
+      <c r="B9" s="15"/>
+    </row>
+    <row r="10" spans="1:2" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A10" s="30" t="s">
+        <v>237</v>
+      </c>
+      <c r="B10" s="15"/>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" s="27" t="s">
+        <v>25</v>
+      </c>
+      <c r="B11" s="15" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="B12" s="28">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" s="12" t="s">
+        <v>184</v>
+      </c>
+      <c r="B13" s="28">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="A14" s="12" t="s">
+        <v>182</v>
+      </c>
+      <c r="B14" s="28">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="A15" s="12" t="s">
+        <v>145</v>
+      </c>
+      <c r="B15" s="28">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16" s="12" t="s">
+        <v>183</v>
+      </c>
+      <c r="B16" s="28">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" s="15" t="s">
+        <v>232</v>
+      </c>
+      <c r="B17" s="28">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" s="15"/>
+      <c r="B18" s="15"/>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" s="15"/>
+      <c r="B19" s="15"/>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A20" s="15"/>
+      <c r="B20" s="15"/>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21" s="15"/>
+      <c r="B21" s="15"/>
+    </row>
+    <row r="22" spans="1:2" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A22" s="30" t="s">
+        <v>238</v>
+      </c>
+      <c r="B22" s="15"/>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A23" s="27" t="s">
+        <v>5</v>
+      </c>
+      <c r="B23" s="15" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A24" s="12" t="s">
+        <v>200</v>
+      </c>
+      <c r="B24" s="28">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A25" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="B25" s="28">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A26" s="12" t="s">
+        <v>187</v>
+      </c>
+      <c r="B26" s="28">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A27" s="12" t="s">
+        <v>153</v>
+      </c>
+      <c r="B27" s="28">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A28" s="12" t="s">
+        <v>234</v>
+      </c>
+      <c r="B28" s="28">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A29" s="15" t="s">
+        <v>232</v>
+      </c>
+      <c r="B29" s="28">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A34" s="30" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A35" s="27" t="s">
+        <v>1</v>
+      </c>
+      <c r="B35" s="15" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A36" s="15" t="s">
+        <v>26</v>
+      </c>
+      <c r="B36" s="29">
+        <v>21215</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A37" s="15" t="s">
+        <v>14</v>
+      </c>
+      <c r="B37" s="29">
+        <v>21480.240624999999</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A38" s="15" t="s">
+        <v>232</v>
+      </c>
+      <c r="B38" s="29">
+        <v>21407.902272727271</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId5"/>
+</worksheet>
 </file>
</xml_diff>